<commit_message>
Fix Summary heterogeneity diagnostics
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -592,34 +592,34 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0.41</v>
+        <v>0.59</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.32</v>
+        <v>0.24</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.53</v>
+        <v>1.43</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.24</v>
+        <v>0.02</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0.71</v>
+        <v>16.99</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>0</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>0.4575581064437775</v>
+        <v>0.8882941697523908</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>3660</v>
+        <v>4428</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>1829</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="5">
@@ -2766,28 +2766,34 @@
         </is>
       </c>
       <c r="B66" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C66" s="5" t="n">
-        <v>1.32</v>
+        <v>1.14</v>
       </c>
       <c r="D66" s="5" t="n">
-        <v>1.12</v>
+        <v>0.8</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="F66" s="5" t="inlineStr"/>
-      <c r="G66" s="5" t="inlineStr"/>
+        <v>1.63</v>
+      </c>
+      <c r="F66" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G66" s="5" t="n">
+        <v>93.62</v>
+      </c>
       <c r="H66" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I66" s="7" t="inlineStr"/>
+        <v>91.5</v>
+      </c>
+      <c r="I66" s="7" t="n">
+        <v>0.214434325667662</v>
+      </c>
       <c r="J66" s="8" t="n">
-        <v>1024</v>
+        <v>4702</v>
       </c>
       <c r="K66" s="8" t="n">
-        <v>417</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="67">

</xml_diff>

<commit_message>
Regenerate summary workbooks and dumbbell plot
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$K$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$K$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -450,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -541,12 +541,12 @@
       <c r="E2" s="5" t="n">
         <v>0.42</v>
       </c>
-      <c r="F2" s="5" t="inlineStr"/>
-      <c r="G2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="n"/>
+      <c r="G2" s="5" t="n"/>
       <c r="H2" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I2" s="7" t="inlineStr"/>
+      <c r="I2" s="7" t="n"/>
       <c r="J2" s="8" t="n">
         <v>305</v>
       </c>
@@ -572,12 +572,12 @@
       <c r="E3" s="5" t="n">
         <v>0.68</v>
       </c>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
       <c r="H3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="7" t="inlineStr"/>
+      <c r="I3" s="7" t="n"/>
       <c r="J3" s="8" t="n">
         <v>415</v>
       </c>
@@ -588,761 +588,767 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>mushrooms</t>
+          <t>cesium</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0.59</v>
+        <v>0.53</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.24</v>
+        <v>0.33</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>1.43</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>16.99</v>
-      </c>
+        <v>0.84</v>
+      </c>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
       <c r="H4" s="6" t="n">
-        <v>91.90000000000001</v>
-      </c>
-      <c r="I4" s="7" t="n">
-        <v>0.8882941697523908</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I4" s="7" t="n"/>
       <c r="J4" s="8" t="n">
-        <v>4428</v>
+        <v>486</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>1957</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>cesium</t>
+          <t>potassium</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.53</v>
+        <v>0.55</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
+        <v>1.03</v>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="7" t="inlineStr"/>
+        <v>74.7</v>
+      </c>
+      <c r="I5" s="7" t="n"/>
       <c r="J5" s="8" t="n">
-        <v>486</v>
+        <v>1370</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>240</v>
+        <v>587</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>potassium</t>
+          <t>molybdenum</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
+        <v>0.96</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>6.78</v>
+      </c>
       <c r="H6" s="6" t="n">
-        <v>74.7</v>
-      </c>
-      <c r="I6" s="7" t="inlineStr"/>
+        <v>94.5</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <v>0.8351773861379137</v>
+      </c>
       <c r="J6" s="8" t="n">
-        <v>1370</v>
+        <v>5809</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>587</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b6</t>
+          <t>papaya</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>0.5600000000000001</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>0.42</v>
+        <v>0.37</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>1.43</v>
-      </c>
+        <v>0.84</v>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
       <c r="H7" s="6" t="n">
-        <v>72.2</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <v>0.006929997867264418</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I7" s="7" t="n"/>
       <c r="J7" s="8" t="n">
-        <v>92079</v>
+        <v>876</v>
       </c>
       <c r="K7" s="8" t="n">
-        <v>3337</v>
+        <v>438</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>papaya</t>
+          <t>mushrooms</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.37</v>
+        <v>0.24</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="5" t="inlineStr"/>
+        <v>1.43</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>16.99</v>
+      </c>
       <c r="H8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="7" t="inlineStr"/>
+        <v>91.90000000000001</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <v>0.8882941697523911</v>
+      </c>
       <c r="J8" s="8" t="n">
-        <v>876</v>
+        <v>4428</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>438</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>molybdenum</t>
+          <t>lutein</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.33</v>
+        <v>0.52</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.96</v>
+        <v>0.72</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.05</v>
+        <v>0.34</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>6.78</v>
+        <v>1.1</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>94.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.8351773861379138</v>
+        <v>0.0003391655256003492</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>5809</v>
+        <v>1073040</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>2459</v>
+        <v>51133</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>legumes</t>
+          <t>vitamin_b6</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>0.5</v>
+        <v>0.44</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.75</v>
+        <v>0.87</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.27</v>
+        <v>0.19</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>1.37</v>
+        <v>1.97</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>94.09999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>0.001758518003460141</v>
+        <v>0.0003230528771021327</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>273560</v>
+        <v>336188</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>15479</v>
+        <v>40095</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>black_cohosh</t>
+          <t>omega-3_fatty_acids</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.61</v>
+        <v>0.65</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.34</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="F11" s="5" t="inlineStr"/>
-      <c r="G11" s="5" t="inlineStr"/>
+        <v>0.76</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>1.17</v>
+      </c>
       <c r="H11" s="6" t="n">
-        <v>76.40000000000001</v>
-      </c>
-      <c r="I11" s="7" t="inlineStr"/>
+        <v>68</v>
+      </c>
+      <c r="I11" s="7" t="n">
+        <v>0.5929735955651932</v>
+      </c>
       <c r="J11" s="8" t="n">
-        <v>12594</v>
+        <v>242088</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>4413</v>
+        <v>10615</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>grape</t>
+          <t>vitamin_b12</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0.62</v>
+        <v>0.66</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.38</v>
+        <v>0.48</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="F12" s="5" t="inlineStr"/>
-      <c r="G12" s="5" t="inlineStr"/>
+        <v>0.91</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>1.9</v>
+      </c>
       <c r="H12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="7" t="inlineStr"/>
+        <v>87.3</v>
+      </c>
+      <c r="I12" s="7" t="n">
+        <v>0.02220092332067387</v>
+      </c>
       <c r="J12" s="8" t="n">
-        <v>1067</v>
+        <v>88794</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>359</v>
+        <v>11404</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>lutein</t>
+          <t>iodine</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.65</v>
+        <v>0.68</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>0.54</v>
+        <v>0.46</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>1.18</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
       <c r="H13" s="6" t="n">
-        <v>79.90000000000001</v>
-      </c>
-      <c r="I13" s="7" t="n">
-        <v>0.009603755584594299</v>
-      </c>
+        <v>44.9</v>
+      </c>
+      <c r="I13" s="7" t="n"/>
       <c r="J13" s="8" t="n">
-        <v>1067447</v>
+        <v>3284</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>48416</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>omega-3_fatty_acids</t>
+          <t>n-acetylcysteine</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>0.65</v>
+        <v>0.7</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.68</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="G14" s="5" t="n">
-        <v>1.17</v>
-      </c>
+        <v>0.73</v>
+      </c>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="6" t="n">
-        <v>68</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>0.5929735955651931</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I14" s="7" t="n"/>
       <c r="J14" s="8" t="n">
-        <v>242088</v>
+        <v>91546</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>10615</v>
+        <v>11901</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b12</t>
+          <t>oats</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0.66</v>
+        <v>0.7</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0.48</v>
+        <v>0.3</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>1.9</v>
-      </c>
+        <v>1.65</v>
+      </c>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
       <c r="H15" s="6" t="n">
-        <v>87.3</v>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>0.02220092332067385</v>
-      </c>
+        <v>82.3</v>
+      </c>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="8" t="n">
-        <v>88794</v>
+        <v>28604</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>11404</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>lycopene</t>
+          <t>garlic</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>0.55</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.84</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.32</v>
+        <v>0.27</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>1.43</v>
+        <v>1.91</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>82.8</v>
+        <v>44.2</v>
       </c>
       <c r="I16" s="7" t="n">
-        <v>0.1176939329825923</v>
+        <v>0.1879066502188127</v>
       </c>
       <c r="J16" s="8" t="n">
-        <v>334206</v>
+        <v>243855</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>132822</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>iodine</t>
+          <t>lycopene</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>0.46</v>
+        <v>0.6</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="5" t="inlineStr"/>
-      <c r="G17" s="5" t="inlineStr"/>
+        <v>0.83</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>1.27</v>
+      </c>
       <c r="H17" s="6" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="I17" s="7" t="inlineStr"/>
+        <v>87.40000000000001</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>0.001143089295674919</v>
+      </c>
       <c r="J17" s="8" t="n">
-        <v>3284</v>
+        <v>370200</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>1288</v>
+        <v>136583</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>n-acetylcysteine</t>
+          <t>antioxidants</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>0.7</v>
+        <v>0.72</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.68</v>
+        <v>0.63</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="5" t="inlineStr"/>
+        <v>0.82</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>1.14</v>
+      </c>
       <c r="H18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" s="7" t="inlineStr"/>
+        <v>85.2</v>
+      </c>
+      <c r="I18" s="7" t="n">
+        <v>0.0009624795570247766</v>
+      </c>
       <c r="J18" s="8" t="n">
-        <v>91546</v>
+        <v>855680</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>11901</v>
+        <v>267009</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>oats</t>
+          <t>beta-carotene</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>0.7</v>
+        <v>0.73</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>0.3</v>
+        <v>0.66</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="F19" s="5" t="inlineStr"/>
-      <c r="G19" s="5" t="inlineStr"/>
+        <v>0.8</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>1.19</v>
+      </c>
       <c r="H19" s="6" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="I19" s="7" t="inlineStr"/>
+        <v>82.90000000000001</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>0.002411799505362666</v>
+      </c>
       <c r="J19" s="8" t="n">
-        <v>28604</v>
+        <v>1817569</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>1075</v>
+        <v>128023</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>garlic</t>
+          <t>mineral_supplements</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.55</v>
+        <v>0.43</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="F20" s="5" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>1.91</v>
-      </c>
+        <v>1.17</v>
+      </c>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
       <c r="H20" s="6" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>0.1879066502188127</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I20" s="7" t="n"/>
       <c r="J20" s="8" t="n">
-        <v>243855</v>
+        <v>836</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>1388</v>
+        <v>312</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>mediterranean_diet</t>
+          <t>black_cohosh</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>0.71</v>
+        <v>0.74</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.79</v>
+        <v>0.92</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.46</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>1.1</v>
+        <v>7.42</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>87.2</v>
+        <v>64.2</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>5.466290886526577e-05</v>
+        <v>0.3220215410089055</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>539860</v>
+        <v>31455</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>28634</v>
+        <v>5515</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>antioxidants</t>
+          <t>legumes</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>0.61</v>
+        <v>0.65</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>1.3</v>
+        <v>1.22</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>84.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>0.022216274500156</v>
+        <v>4.315818448979679e-05</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>856523</v>
+        <v>273560</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>267423</v>
+        <v>15479</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>soy</t>
+          <t>olive</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="C23" s="5" t="n">
-        <v>0.73</v>
+        <v>0.75</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.31</v>
+        <v>0.45</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>1.69</v>
+        <v>1.24</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>90.59999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.01141221985751853</v>
+        <v>0.005850985088450084</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>959523</v>
+        <v>249237</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>33957</v>
+        <v>17161</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b1</t>
+          <t>soy</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>0.75</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>0.61</v>
+        <v>0.65</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="F24" s="5" t="inlineStr"/>
-      <c r="G24" s="5" t="inlineStr"/>
+        <v>0.86</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>1.75</v>
+      </c>
       <c r="H24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="7" t="inlineStr"/>
+        <v>90.8</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>0.02203868687349753</v>
+      </c>
       <c r="J24" s="8" t="n">
-        <v>38639</v>
+        <v>961262</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>853</v>
+        <v>34226</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>fish_oil</t>
+          <t>vitamin_b1</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>2.06</v>
-      </c>
+        <v>0.93</v>
+      </c>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
       <c r="H25" s="6" t="n">
-        <v>82.40000000000001</v>
-      </c>
-      <c r="I25" s="7" t="n">
-        <v>0.02000889385459846</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I25" s="7" t="n"/>
       <c r="J25" s="8" t="n">
-        <v>508427</v>
+        <v>38639</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>63225</v>
+        <v>853</v>
       </c>
     </row>
     <row r="26">
@@ -1373,7 +1379,7 @@
         <v>90.5</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>0.1085966579317358</v>
+        <v>0.1085966579317357</v>
       </c>
       <c r="J26" s="8" t="n">
         <v>80262</v>
@@ -1385,106 +1391,112 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>beta-carotene</t>
+          <t>fish_oil</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="C27" s="5" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>0.68</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>0.89</v>
+        <v>1.02</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.38</v>
+        <v>0.28</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>1.56</v>
+        <v>2.06</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>89.40000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.09603493939892245</v>
+        <v>0.02000889385459848</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>1382343</v>
+        <v>508427</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>76186</v>
+        <v>63225</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>betaine</t>
+          <t>mediterranean_diet</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>1.07</v>
+        <v>0.83</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.02</v>
+        <v>0.54</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>37.25</v>
+        <v>1.08</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>81.90000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>0.177930339763042</v>
+        <v>4.147592651637327e-05</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>77198</v>
+        <v>639823</v>
       </c>
       <c r="K28" s="8" t="n">
-        <v>5297</v>
+        <v>40922</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>bcaas</t>
+          <t>betaine</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>0.77</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>0.4</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="F29" s="5" t="inlineStr"/>
-      <c r="G29" s="5" t="inlineStr"/>
+        <v>1.07</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>37.25</v>
+      </c>
       <c r="H29" s="6" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="I29" s="7" t="inlineStr"/>
+        <v>81.90000000000001</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>0.1779303397630421</v>
+      </c>
       <c r="J29" s="8" t="n">
-        <v>197211</v>
+        <v>77198</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>10396</v>
+        <v>5297</v>
       </c>
     </row>
     <row r="30">
@@ -1505,12 +1517,12 @@
       <c r="E30" s="5" t="n">
         <v>0.9</v>
       </c>
-      <c r="F30" s="5" t="inlineStr"/>
-      <c r="G30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
       <c r="H30" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I30" s="7" t="inlineStr"/>
+      <c r="I30" s="7" t="n"/>
       <c r="J30" s="8" t="n">
         <v>4001</v>
       </c>
@@ -1521,38 +1533,38 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>olive</t>
+          <t>folic_acid</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.72</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.92</v>
+        <v>0.88</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.51</v>
+        <v>0.47</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>1.24</v>
+        <v>1.35</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>81</v>
+        <v>81.5</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.01389915282783273</v>
+        <v>0.001821422591105356</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>248595</v>
+        <v>1079347</v>
       </c>
       <c r="K31" s="8" t="n">
-        <v>16870</v>
+        <v>52296</v>
       </c>
     </row>
     <row r="32">
@@ -1583,7 +1595,7 @@
         <v>57</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>0.5607534123225345</v>
+        <v>0.5607534123225346</v>
       </c>
       <c r="J32" s="8" t="n">
         <v>87065</v>
@@ -1620,7 +1632,7 @@
         <v>90.8</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.5897124894853762</v>
+        <v>0.5897124894853758</v>
       </c>
       <c r="J33" s="8" t="n">
         <v>190614</v>
@@ -1632,38 +1644,38 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>folic_acid</t>
+          <t>vitamin_e</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>0.82</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.46</v>
+        <v>0.41</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>1.48</v>
+        <v>1.65</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>84.5</v>
+        <v>85</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.02877266109333391</v>
+        <v>0.2610709779752496</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>1079462</v>
+        <v>558626</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>52354</v>
+        <v>157061</v>
       </c>
     </row>
     <row r="35">
@@ -1694,7 +1706,7 @@
         <v>58.7</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.0321383112172301</v>
+        <v>0.03213831121723015</v>
       </c>
       <c r="J35" s="8" t="n">
         <v>20962</v>
@@ -1706,44 +1718,38 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>vitamin_d</t>
+          <t>flax</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>79</v>
+        <v>1</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>0.84</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>0.8</v>
+        <v>0.72</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="F36" s="5" t="n">
-        <v>0.64</v>
-      </c>
-      <c r="G36" s="5" t="n">
-        <v>1.09</v>
-      </c>
+        <v>0.97</v>
+      </c>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
       <c r="H36" s="6" t="n">
-        <v>84.2</v>
-      </c>
-      <c r="I36" s="7" t="n">
-        <v>2.803290338106087e-10</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I36" s="7" t="n"/>
       <c r="J36" s="8" t="n">
-        <v>1568014</v>
+        <v>6369</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>240492</v>
+        <v>2999</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>flax</t>
+          <t>flaxseed</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
@@ -1758,12 +1764,12 @@
       <c r="E37" s="5" t="n">
         <v>0.97</v>
       </c>
-      <c r="F37" s="5" t="inlineStr"/>
-      <c r="G37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
       <c r="H37" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="7" t="inlineStr"/>
+      <c r="I37" s="7" t="n"/>
       <c r="J37" s="8" t="n">
         <v>6369</v>
       </c>
@@ -1774,32 +1780,38 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>flaxseed</t>
+          <t>vitamin_d</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>1</v>
+        <v>79</v>
       </c>
       <c r="C38" s="5" t="n">
         <v>0.84</v>
       </c>
       <c r="D38" s="5" t="n">
-        <v>0.72</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="F38" s="5" t="inlineStr"/>
-      <c r="G38" s="5" t="inlineStr"/>
+        <v>0.88</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>1.1</v>
+      </c>
       <c r="H38" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" s="7" t="inlineStr"/>
+        <v>84.09999999999999</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>3.89041909401795e-09</v>
+      </c>
       <c r="J38" s="8" t="n">
-        <v>6369</v>
+        <v>1568223</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>2999</v>
+        <v>240235</v>
       </c>
     </row>
     <row r="39">
@@ -1820,12 +1832,12 @@
       <c r="E39" s="5" t="n">
         <v>0.99</v>
       </c>
-      <c r="F39" s="5" t="inlineStr"/>
-      <c r="G39" s="5" t="inlineStr"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
       <c r="H39" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="7" t="inlineStr"/>
+      <c r="I39" s="7" t="n"/>
       <c r="J39" s="8" t="n">
         <v>2939</v>
       </c>
@@ -1840,182 +1852,182 @@
         </is>
       </c>
       <c r="B40" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>0.87</v>
+        <v>0.85</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>0.73</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>1.03</v>
+        <v>1</v>
       </c>
       <c r="F40" s="5" t="n">
         <v>0.55</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>1.38</v>
+        <v>1.31</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>45.5</v>
+        <v>42.3</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>0.8096930861186751</v>
+        <v>0.9864318175325136</v>
       </c>
       <c r="J40" s="8" t="n">
-        <v>28894</v>
+        <v>62422</v>
       </c>
       <c r="K40" s="8" t="n">
-        <v>2650</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>vitamin_a</t>
+          <t>green_tea</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>0.9</v>
+        <v>0.89</v>
       </c>
       <c r="D41" s="5" t="n">
-        <v>0.74</v>
+        <v>0.77</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>1.08</v>
+        <v>1.02</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.44</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>1.84</v>
+        <v>1.4</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>86</v>
+        <v>85.7</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.4943075797793355</v>
+        <v>0.192122449317125</v>
       </c>
       <c r="J41" s="8" t="n">
-        <v>551013</v>
+        <v>274406</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>143360</v>
+        <v>18211</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>calcium</t>
+          <t>vitamin_a</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>0.92</v>
+        <v>0.9</v>
       </c>
       <c r="D42" s="5" t="n">
-        <v>0.87</v>
+        <v>0.74</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.96</v>
+        <v>1.08</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.79</v>
+        <v>0.44</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>1.06</v>
+        <v>1.84</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>77.7</v>
+        <v>86</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>0.004434867735702238</v>
+        <v>0.4943075797793356</v>
       </c>
       <c r="J42" s="8" t="n">
-        <v>893832</v>
+        <v>551013</v>
       </c>
       <c r="K42" s="8" t="n">
-        <v>76347</v>
+        <v>143360</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>vitamin_c</t>
+          <t>calcium</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="D43" s="5" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>1.06</v>
+        <v>0.96</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0.59</v>
+        <v>0.76</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>1.48</v>
+        <v>1.08</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>0.5612991451474079</v>
+        <v>0.02639264973927776</v>
       </c>
       <c r="J43" s="8" t="n">
-        <v>512782</v>
+        <v>894018</v>
       </c>
       <c r="K43" s="8" t="n">
-        <v>35415</v>
+        <v>76477</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>vitamin_e</t>
+          <t>vitamin_c</t>
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C44" s="5" t="n">
         <v>0.9399999999999999</v>
       </c>
       <c r="D44" s="5" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.82</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>1.1</v>
+        <v>1.06</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.5</v>
+        <v>0.59</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>1.79</v>
+        <v>1.48</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>84.2</v>
+        <v>83</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>0.9988584509209855</v>
+        <v>0.5612991451474082</v>
       </c>
       <c r="J44" s="8" t="n">
-        <v>717001</v>
+        <v>512782</v>
       </c>
       <c r="K44" s="8" t="n">
-        <v>276935</v>
+        <v>35415</v>
       </c>
     </row>
     <row r="45">
@@ -2025,108 +2037,108 @@
         </is>
       </c>
       <c r="B45" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="D45" s="5" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>1.05</v>
+        <v>1.03</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>1.23</v>
+        <v>1.22</v>
       </c>
       <c r="H45" s="6" t="n">
         <v>58.4</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>0.9919383665571089</v>
+        <v>0.8524602198215492</v>
       </c>
       <c r="J45" s="8" t="n">
-        <v>343803</v>
+        <v>346098</v>
       </c>
       <c r="K45" s="8" t="n">
-        <v>20200</v>
+        <v>21359</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>green_tea</t>
+          <t>caffeine</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C46" s="5" t="n">
         <v>0.97</v>
       </c>
       <c r="D46" s="5" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="E46" s="5" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F46" s="5" t="n">
         <v>0.85</v>
       </c>
-      <c r="E46" s="5" t="n">
+      <c r="G46" s="5" t="n">
         <v>1.1</v>
       </c>
-      <c r="F46" s="5" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="G46" s="5" t="n">
-        <v>1.4</v>
-      </c>
       <c r="H46" s="6" t="n">
-        <v>74.5</v>
+        <v>45.9</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0.4286050916258499</v>
+        <v>0.4259906328747247</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>233848</v>
+        <v>872194</v>
       </c>
       <c r="K46" s="8" t="n">
-        <v>16921</v>
+        <v>38461</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>caffeine</t>
+          <t>bcaas</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>0.92</v>
+        <v>0.87</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>1.01</v>
+        <v>1.11</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.85</v>
+        <v>0.63</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1.1</v>
+        <v>1.55</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>45.9</v>
+        <v>79.5</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>0.4259906328747249</v>
+        <v>0.5438582918197439</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>872194</v>
+        <v>224226</v>
       </c>
       <c r="K47" s="8" t="n">
-        <v>38461</v>
+        <v>14045</v>
       </c>
     </row>
     <row r="48">
@@ -2136,34 +2148,34 @@
         </is>
       </c>
       <c r="B48" s="4" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="D48" s="5" t="n">
-        <v>0.95</v>
+        <v>0.96</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>85.2</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>0.2491322927934893</v>
+        <v>0.314801545381515</v>
       </c>
       <c r="J48" s="8" t="n">
-        <v>2737742</v>
+        <v>2900381</v>
       </c>
       <c r="K48" s="8" t="n">
-        <v>194366</v>
+        <v>201856</v>
       </c>
     </row>
     <row r="49">
@@ -2194,7 +2206,7 @@
         <v>86.09999999999999</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>0.9376775415524332</v>
+        <v>0.9376775415524331</v>
       </c>
       <c r="J49" s="8" t="n">
         <v>227916</v>
@@ -2206,625 +2218,625 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>vitamin_k</t>
+          <t>leucine</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C50" s="5" t="n">
         <v>1.01</v>
       </c>
       <c r="D50" s="5" t="n">
-        <v>0.68</v>
+        <v>0.91</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F50" s="5" t="inlineStr"/>
-      <c r="G50" s="5" t="inlineStr"/>
+        <v>1.13</v>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>1.57</v>
+      </c>
       <c r="H50" s="6" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="I50" s="7" t="inlineStr"/>
+        <v>80.8</v>
+      </c>
+      <c r="I50" s="7" t="n">
+        <v>0.5613202208181793</v>
+      </c>
       <c r="J50" s="8" t="n">
-        <v>5048</v>
+        <v>225687</v>
       </c>
       <c r="K50" s="8" t="n">
-        <v>2592</v>
+        <v>15633</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>tea</t>
+          <t>vitamin_k</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="C51" s="5" t="n">
-        <v>1.04</v>
+        <v>1.01</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>0.99</v>
+        <v>0.68</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="F51" s="5" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G51" s="5" t="n">
-        <v>1.19</v>
-      </c>
+        <v>1.5</v>
+      </c>
+      <c r="F51" s="5" t="n"/>
+      <c r="G51" s="5" t="n"/>
       <c r="H51" s="6" t="n">
-        <v>90.40000000000001</v>
-      </c>
-      <c r="I51" s="7" t="n">
-        <v>0.804669086136711</v>
-      </c>
+        <v>91.8</v>
+      </c>
+      <c r="I51" s="7" t="n"/>
       <c r="J51" s="8" t="n">
-        <v>1885475</v>
+        <v>5048</v>
       </c>
       <c r="K51" s="8" t="n">
-        <v>231699</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>conjugated_linoleic_acid</t>
+          <t>tea</t>
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="C52" s="5" t="n">
-        <v>1.06</v>
+        <v>1.02</v>
       </c>
       <c r="D52" s="5" t="n">
-        <v>0.92</v>
+        <v>0.95</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0.62</v>
+        <v>0.74</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>1.82</v>
+        <v>1.4</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>62</v>
+        <v>90.5</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>0.4225544208553845</v>
+        <v>0.8887019962528848</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>380443</v>
+        <v>1885475</v>
       </c>
       <c r="K52" s="8" t="n">
-        <v>17329</v>
+        <v>231699</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>glucosamine</t>
+          <t>carnitine</t>
         </is>
       </c>
       <c r="B53" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C53" s="5" t="n">
-        <v>1.06</v>
+        <v>1.03</v>
       </c>
       <c r="D53" s="5" t="n">
-        <v>0.93</v>
+        <v>0.82</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="F53" s="5" t="inlineStr"/>
-      <c r="G53" s="5" t="inlineStr"/>
+        <v>1.3</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>2.45</v>
+      </c>
       <c r="H53" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" s="7" t="inlineStr"/>
+        <v>91.09999999999999</v>
+      </c>
+      <c r="I53" s="7" t="n">
+        <v>0.8134382130434087</v>
+      </c>
       <c r="J53" s="8" t="n">
-        <v>41082</v>
+        <v>800654</v>
       </c>
       <c r="K53" s="8" t="n">
-        <v>5341</v>
+        <v>194212</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>leucine</t>
+          <t>quercetin</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="5" t="n">
-        <v>1.07</v>
+        <v>1.05</v>
       </c>
       <c r="D54" s="5" t="n">
-        <v>0.95</v>
+        <v>0.83</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F54" s="5" t="inlineStr"/>
-      <c r="G54" s="5" t="inlineStr"/>
+        <v>1.34</v>
+      </c>
+      <c r="F54" s="5" t="n"/>
+      <c r="G54" s="5" t="n"/>
       <c r="H54" s="6" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="I54" s="7" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="I54" s="7" t="n"/>
       <c r="J54" s="8" t="n">
-        <v>28476</v>
+        <v>90630</v>
       </c>
       <c r="K54" s="8" t="n">
-        <v>5237</v>
+        <v>710</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>grapefruit</t>
+          <t>conjugated_linoleic_acid</t>
         </is>
       </c>
       <c r="B55" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C55" s="5" t="n">
-        <v>1.1</v>
+        <v>1.06</v>
       </c>
       <c r="D55" s="5" t="n">
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>1.52</v>
-      </c>
-      <c r="F55" s="5" t="inlineStr"/>
-      <c r="G55" s="5" t="inlineStr"/>
+        <v>1.22</v>
+      </c>
+      <c r="F55" s="5" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G55" s="5" t="n">
+        <v>1.82</v>
+      </c>
       <c r="H55" s="6" t="n">
-        <v>82.8</v>
-      </c>
-      <c r="I55" s="7" t="inlineStr"/>
+        <v>62</v>
+      </c>
+      <c r="I55" s="7" t="n">
+        <v>0.4225544208553845</v>
+      </c>
       <c r="J55" s="8" t="n">
-        <v>164504</v>
+        <v>380443</v>
       </c>
       <c r="K55" s="8" t="n">
-        <v>5404</v>
+        <v>17329</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>creatine</t>
+          <t>glucosamine</t>
         </is>
       </c>
       <c r="B56" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C56" s="5" t="n">
-        <v>1.11</v>
+        <v>1.06</v>
       </c>
       <c r="D56" s="5" t="n">
-        <v>1.01</v>
+        <v>0.93</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="F56" s="5" t="inlineStr"/>
-      <c r="G56" s="5" t="inlineStr"/>
+        <v>1.21</v>
+      </c>
+      <c r="F56" s="5" t="n"/>
+      <c r="G56" s="5" t="n"/>
       <c r="H56" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I56" s="7" t="inlineStr"/>
+      <c r="I56" s="7" t="n"/>
       <c r="J56" s="8" t="n">
-        <v>207</v>
+        <v>41082</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>1057</v>
+        <v>5341</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>carnitine</t>
+          <t>grape</t>
         </is>
       </c>
       <c r="B57" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C57" s="5" t="n">
-        <v>1.13</v>
+        <v>1.08</v>
       </c>
       <c r="D57" s="5" t="n">
-        <v>0.9</v>
+        <v>0.36</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="F57" s="5" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="G57" s="5" t="n">
-        <v>3.02</v>
-      </c>
+        <v>3.21</v>
+      </c>
+      <c r="F57" s="5" t="n"/>
+      <c r="G57" s="5" t="n"/>
       <c r="H57" s="6" t="n">
-        <v>82.8</v>
-      </c>
-      <c r="I57" s="7" t="n">
-        <v>0.7636681889414908</v>
-      </c>
+        <v>89.3</v>
+      </c>
+      <c r="I57" s="7" t="n"/>
       <c r="J57" s="8" t="n">
-        <v>384266</v>
+        <v>1816</v>
       </c>
       <c r="K57" s="8" t="n">
-        <v>140082</v>
+        <v>609</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>chromium</t>
+          <t>magnesium</t>
         </is>
       </c>
       <c r="B58" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C58" s="5" t="n">
-        <v>1.13</v>
+        <v>1.08</v>
       </c>
       <c r="D58" s="5" t="n">
-        <v>1.06</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>1.21</v>
+        <v>1.25</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>0.74</v>
+        <v>0.66</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>1.74</v>
+        <v>1.78</v>
       </c>
       <c r="H58" s="6" t="n">
-        <v>0</v>
+        <v>93</v>
       </c>
       <c r="I58" s="7" t="n">
-        <v>0.987786419099957</v>
+        <v>0.4685196145888207</v>
       </c>
       <c r="J58" s="8" t="n">
-        <v>66508</v>
+        <v>1239364</v>
       </c>
       <c r="K58" s="8" t="n">
-        <v>1506</v>
+        <v>266355</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>magnesium</t>
+          <t>coenzyme_q10</t>
         </is>
       </c>
       <c r="B59" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C59" s="5" t="n">
-        <v>1.13</v>
+        <v>1.1</v>
       </c>
       <c r="D59" s="5" t="n">
-        <v>0.97</v>
+        <v>0.36</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="F59" s="5" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="G59" s="5" t="n">
-        <v>2.19</v>
-      </c>
+        <v>3.34</v>
+      </c>
+      <c r="F59" s="5" t="n"/>
+      <c r="G59" s="5" t="n"/>
       <c r="H59" s="6" t="n">
-        <v>83.8</v>
-      </c>
-      <c r="I59" s="7" t="n">
-        <v>0.9619708795552824</v>
-      </c>
+        <v>91.59999999999999</v>
+      </c>
+      <c r="I59" s="7" t="n"/>
       <c r="J59" s="8" t="n">
-        <v>1172319</v>
+        <v>3633</v>
       </c>
       <c r="K59" s="8" t="n">
-        <v>257639</v>
+        <v>725</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>zinc</t>
+          <t>grapefruit</t>
         </is>
       </c>
       <c r="B60" s="4" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C60" s="5" t="n">
-        <v>1.14</v>
+        <v>1.1</v>
       </c>
       <c r="D60" s="5" t="n">
-        <v>0.68</v>
+        <v>0.8</v>
       </c>
       <c r="E60" s="5" t="n">
-        <v>1.91</v>
-      </c>
-      <c r="F60" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="G60" s="5" t="n">
-        <v>8.09</v>
-      </c>
+        <v>1.52</v>
+      </c>
+      <c r="F60" s="5" t="n"/>
+      <c r="G60" s="5" t="n"/>
       <c r="H60" s="6" t="n">
-        <v>96</v>
-      </c>
-      <c r="I60" s="7" t="n">
-        <v>0.6073544042976847</v>
-      </c>
+        <v>82.8</v>
+      </c>
+      <c r="I60" s="7" t="n"/>
       <c r="J60" s="8" t="n">
-        <v>119440</v>
+        <v>164504</v>
       </c>
       <c r="K60" s="8" t="n">
-        <v>10103</v>
+        <v>5404</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>iron</t>
+          <t>creatine</t>
         </is>
       </c>
       <c r="B61" s="4" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C61" s="5" t="n">
-        <v>1.15</v>
+        <v>1.11</v>
       </c>
       <c r="D61" s="5" t="n">
-        <v>1.06</v>
+        <v>1.01</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="F61" s="5" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="G61" s="5" t="n">
-        <v>1.58</v>
-      </c>
+        <v>1.19</v>
+      </c>
+      <c r="F61" s="5" t="n"/>
+      <c r="G61" s="5" t="n"/>
       <c r="H61" s="6" t="n">
-        <v>80.59999999999999</v>
-      </c>
-      <c r="I61" s="7" t="n">
-        <v>0.1723925153093609</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I61" s="7" t="n"/>
       <c r="J61" s="8" t="n">
-        <v>1376214</v>
+        <v>207</v>
       </c>
       <c r="K61" s="8" t="n">
-        <v>221434</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>eggs</t>
+          <t>chromium</t>
         </is>
       </c>
       <c r="B62" s="4" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="C62" s="5" t="n">
-        <v>1.15</v>
+        <v>1.13</v>
       </c>
       <c r="D62" s="5" t="n">
-        <v>0.95</v>
+        <v>1.06</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>1.39</v>
+        <v>1.21</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>0.67</v>
+        <v>0.74</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>1.96</v>
+        <v>1.74</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>86.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>0.7478766568479693</v>
+        <v>0.9877864190999566</v>
       </c>
       <c r="J62" s="8" t="n">
-        <v>29487</v>
+        <v>66508</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>5481</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>red_meat</t>
+          <t>glutamine</t>
         </is>
       </c>
       <c r="B63" s="4" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="C63" s="5" t="n">
-        <v>1.26</v>
+        <v>1.14</v>
       </c>
       <c r="D63" s="5" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>1.34</v>
+        <v>1.63</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>1</v>
+        <v>0.01</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>1.6</v>
+        <v>93.62</v>
       </c>
       <c r="H63" s="6" t="n">
-        <v>88.40000000000001</v>
+        <v>91.5</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>3.550216935243029e-10</v>
+        <v>0.214434325667662</v>
       </c>
       <c r="J63" s="8" t="n">
-        <v>1188831</v>
+        <v>4702</v>
       </c>
       <c r="K63" s="8" t="n">
-        <v>70016</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>dehydroepiandrosterone</t>
+          <t>zinc</t>
         </is>
       </c>
       <c r="B64" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C64" s="5" t="n">
-        <v>1.27</v>
+        <v>1.14</v>
       </c>
       <c r="D64" s="5" t="n">
-        <v>1.16</v>
+        <v>0.68</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>1.4</v>
+        <v>1.91</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>0.97</v>
+        <v>0.16</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>1.68</v>
+        <v>8.09</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>65.3</v>
+        <v>96</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>0.0001090796573211561</v>
+        <v>0.6073544042976849</v>
       </c>
       <c r="J64" s="8" t="n">
-        <v>248188</v>
+        <v>119440</v>
       </c>
       <c r="K64" s="8" t="n">
-        <v>127366</v>
+        <v>10103</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>phosphorus</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="B65" s="4" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="C65" s="5" t="n">
-        <v>1.27</v>
+        <v>1.15</v>
       </c>
       <c r="D65" s="5" t="n">
-        <v>0.49</v>
+        <v>1.06</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="F65" s="5" t="inlineStr"/>
-      <c r="G65" s="5" t="inlineStr"/>
+        <v>1.25</v>
+      </c>
+      <c r="F65" s="5" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G65" s="5" t="n">
+        <v>1.58</v>
+      </c>
       <c r="H65" s="6" t="n">
-        <v>78.2</v>
-      </c>
-      <c r="I65" s="7" t="inlineStr"/>
+        <v>80.59999999999999</v>
+      </c>
+      <c r="I65" s="7" t="n">
+        <v>0.1723925153093608</v>
+      </c>
       <c r="J65" s="8" t="n">
-        <v>229321</v>
+        <v>1376214</v>
       </c>
       <c r="K65" s="8" t="n">
-        <v>123051</v>
+        <v>221434</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>glutamine</t>
+          <t>eggs</t>
         </is>
       </c>
       <c r="B66" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C66" s="5" t="n">
-        <v>1.14</v>
+        <v>1.19</v>
       </c>
       <c r="D66" s="5" t="n">
-        <v>0.8</v>
+        <v>0.99</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>1.63</v>
+        <v>1.43</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>0.01</v>
+        <v>0.7</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>93.62</v>
+        <v>2.02</v>
       </c>
       <c r="H66" s="6" t="n">
-        <v>91.5</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>0.214434325667662</v>
+        <v>0.9936223155021588</v>
       </c>
       <c r="J66" s="8" t="n">
-        <v>4702</v>
+        <v>29311</v>
       </c>
       <c r="K66" s="8" t="n">
-        <v>2112</v>
+        <v>5421</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>cannabidiol</t>
+          <t>dehydroepiandrosterone</t>
         </is>
       </c>
       <c r="B67" s="4" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C67" s="5" t="n">
-        <v>1.4</v>
+        <v>1.25</v>
       </c>
       <c r="D67" s="5" t="n">
-        <v>1.39</v>
+        <v>1.15</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F67" s="5" t="inlineStr"/>
-      <c r="G67" s="5" t="inlineStr"/>
+        <v>1.36</v>
+      </c>
+      <c r="F67" s="5" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G67" s="5" t="n">
+        <v>1.61</v>
+      </c>
       <c r="H67" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I67" s="7" t="inlineStr"/>
+        <v>62.7</v>
+      </c>
+      <c r="I67" s="7" t="n">
+        <v>6.586804402476428e-05</v>
+      </c>
       <c r="J67" s="8" t="n">
-        <v>124896418350</v>
+        <v>249396</v>
       </c>
       <c r="K67" s="8" t="n">
-        <v>51623922</v>
+        <v>127523</v>
       </c>
     </row>
     <row r="68">
@@ -2834,174 +2846,242 @@
         </is>
       </c>
       <c r="B68" s="4" t="n">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="C68" s="5" t="n">
-        <v>1.38</v>
+        <v>1.26</v>
       </c>
       <c r="D68" s="5" t="n">
-        <v>1.33</v>
+        <v>1.23</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>1.44</v>
+        <v>1.29</v>
       </c>
       <c r="F68" s="5" t="n">
-        <v>0.87</v>
+        <v>1.05</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>2.2</v>
+        <v>1.52</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>98.2</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>5.91216845462099e-07</v>
+        <v>8.11707600187357e-33</v>
       </c>
       <c r="J68" s="8" t="n">
-        <v>17027950</v>
+        <v>16482295</v>
       </c>
       <c r="K68" s="8" t="n">
-        <v>1688752</v>
+        <v>1437638</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>copper</t>
+          <t>phosphorus</t>
         </is>
       </c>
       <c r="B69" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C69" s="5" t="n">
-        <v>1.49</v>
+        <v>1.27</v>
       </c>
       <c r="D69" s="5" t="n">
-        <v>0.95</v>
+        <v>0.49</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>2.31</v>
-      </c>
-      <c r="F69" s="5" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="G69" s="5" t="n">
-        <v>6.92</v>
-      </c>
+        <v>3.26</v>
+      </c>
+      <c r="F69" s="5" t="n"/>
+      <c r="G69" s="5" t="n"/>
       <c r="H69" s="6" t="n">
-        <v>87.3</v>
-      </c>
-      <c r="I69" s="7" t="n">
-        <v>0.6033187907654798</v>
-      </c>
+        <v>78.2</v>
+      </c>
+      <c r="I69" s="7" t="n"/>
       <c r="J69" s="8" t="n">
-        <v>65169</v>
+        <v>229321</v>
       </c>
       <c r="K69" s="8" t="n">
-        <v>1638</v>
+        <v>123051</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>omega-6_fatty_acids</t>
+          <t>red_meat</t>
         </is>
       </c>
       <c r="B70" s="4" t="n">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="C70" s="5" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="D70" s="5" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E70" s="5" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F70" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="5" t="n">
         <v>1.61</v>
       </c>
-      <c r="D70" s="5" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="E70" s="5" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="F70" s="5" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="G70" s="5" t="n">
-        <v>5.26</v>
-      </c>
       <c r="H70" s="6" t="n">
-        <v>50.2</v>
+        <v>88.3</v>
       </c>
       <c r="I70" s="7" t="n">
-        <v>0.04297484100725812</v>
+        <v>1.319761565701648e-10</v>
       </c>
       <c r="J70" s="8" t="n">
-        <v>6123</v>
+        <v>1260095</v>
       </c>
       <c r="K70" s="8" t="n">
-        <v>2981</v>
+        <v>70729</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>coenzyme_q10</t>
+          <t>cannabidiol</t>
         </is>
       </c>
       <c r="B71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="C71" s="5" t="n">
-        <v>1.94</v>
+        <v>1.4</v>
       </c>
       <c r="D71" s="5" t="n">
-        <v>1.19</v>
+        <v>1.39</v>
       </c>
       <c r="E71" s="5" t="n">
-        <v>2.96</v>
-      </c>
-      <c r="F71" s="5" t="inlineStr"/>
-      <c r="G71" s="5" t="inlineStr"/>
+        <v>1.4</v>
+      </c>
+      <c r="F71" s="5" t="n"/>
+      <c r="G71" s="5" t="n"/>
       <c r="H71" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I71" s="7" t="inlineStr"/>
+      <c r="I71" s="7" t="n"/>
       <c r="J71" s="8" t="n">
-        <v>449</v>
+        <v>124896418350</v>
       </c>
       <c r="K71" s="8" t="n">
-        <v>160</v>
+        <v>51623922</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
+          <t>copper</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C72" s="5" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="D72" s="5" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E72" s="5" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="F72" s="5" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G72" s="5" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H72" s="6" t="n">
+        <v>89</v>
+      </c>
+      <c r="I72" s="7" t="n">
+        <v>0.4612984675749361</v>
+      </c>
+      <c r="J72" s="8" t="n">
+        <v>65747</v>
+      </c>
+      <c r="K72" s="8" t="n">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>omega-6_fatty_acids</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C73" s="5" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="D73" s="5" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="E73" s="5" t="n">
+        <v>2.51</v>
+      </c>
+      <c r="F73" s="5" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="G73" s="5" t="n">
+        <v>12.25</v>
+      </c>
+      <c r="H73" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="7" t="n">
+        <v>0.3558547673635933</v>
+      </c>
+      <c r="J73" s="8" t="n">
+        <v>3160</v>
+      </c>
+      <c r="K73" s="8" t="n">
+        <v>1518</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
           <t>pickled_vegetables</t>
         </is>
       </c>
-      <c r="B72" s="4" t="n">
+      <c r="B74" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C72" s="5" t="n">
+      <c r="C74" s="5" t="n">
         <v>3.71</v>
       </c>
-      <c r="D72" s="5" t="n">
+      <c r="D74" s="5" t="n">
         <v>2.67</v>
       </c>
-      <c r="E72" s="5" t="n">
+      <c r="E74" s="5" t="n">
         <v>4.78</v>
       </c>
-      <c r="F72" s="5" t="inlineStr"/>
-      <c r="G72" s="5" t="inlineStr"/>
-      <c r="H72" s="6" t="n">
+      <c r="F74" s="5" t="n"/>
+      <c r="G74" s="5" t="n"/>
+      <c r="H74" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I72" s="7" t="inlineStr"/>
-      <c r="J72" s="8" t="n">
+      <c r="I74" s="7" t="n"/>
+      <c r="J74" s="8" t="n">
         <v>718</v>
       </c>
-      <c r="K72" s="8" t="n">
+      <c r="K74" s="8" t="n">
         <v>358</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K72"/>
+  <autoFilter ref="A1:K74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh multilingual summary plots from current inclusions
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -675,7 +675,7 @@
         <v>94.5</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>0.8351773861379137</v>
+        <v>0.8351773861379138</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>5809</v>
@@ -743,7 +743,7 @@
         <v>91.90000000000001</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.8882941697523911</v>
+        <v>0.8882941697523908</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>4428</v>
@@ -759,34 +759,34 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.61</v>
+        <v>0.62</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>0.52</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>79.09999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.0003391655256003492</v>
+        <v>0.0008471154848143979</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>1073040</v>
+        <v>1072840</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>51133</v>
+        <v>51083</v>
       </c>
     </row>
     <row r="10">
@@ -817,7 +817,7 @@
         <v>86.09999999999999</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>0.0003230528771021327</v>
+        <v>0.0003230528771021325</v>
       </c>
       <c r="J10" s="8" t="n">
         <v>336188</v>
@@ -829,75 +829,75 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>omega-3_fatty_acids</t>
+          <t>vitamin_b12</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.48</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.76</v>
+        <v>0.91</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.36</v>
+        <v>0.23</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>1.17</v>
+        <v>1.9</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>68</v>
+        <v>87.3</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.5929735955651932</v>
+        <v>0.02220092332067385</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>242088</v>
+        <v>88794</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>10615</v>
+        <v>11404</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b12</t>
+          <t>omega-3_fatty_acids</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.48</v>
+        <v>0.58</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.23</v>
+        <v>0.36</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>1.9</v>
+        <v>1.24</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>87.3</v>
+        <v>71.5</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>0.02220092332067387</v>
+        <v>0.4514368397136518</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>88794</v>
+        <v>267959</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>11404</v>
+        <v>13978</v>
       </c>
     </row>
     <row r="13">
@@ -1058,7 +1058,7 @@
         <v>87.40000000000001</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>0.001143089295674919</v>
+        <v>0.001143089295674924</v>
       </c>
       <c r="J17" s="8" t="n">
         <v>370200</v>
@@ -1095,7 +1095,7 @@
         <v>85.2</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>0.0009624795570247766</v>
+        <v>0.0009624795570247788</v>
       </c>
       <c r="J18" s="8" t="n">
         <v>855680</v>
@@ -1132,7 +1132,7 @@
         <v>82.90000000000001</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.002411799505362666</v>
+        <v>0.002411799505362664</v>
       </c>
       <c r="J19" s="8" t="n">
         <v>1817569</v>
@@ -1200,7 +1200,7 @@
         <v>64.2</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3220215410089055</v>
+        <v>0.3220215410089056</v>
       </c>
       <c r="J21" s="8" t="n">
         <v>31455</v>
@@ -1237,7 +1237,7 @@
         <v>86.09999999999999</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>4.315818448979679e-05</v>
+        <v>4.31581844897966e-05</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>273560</v>
@@ -1274,7 +1274,7 @@
         <v>84.8</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.005850985088450084</v>
+        <v>0.005850985088450085</v>
       </c>
       <c r="J23" s="8" t="n">
         <v>249237</v>
@@ -1311,7 +1311,7 @@
         <v>90.8</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>0.02203868687349753</v>
+        <v>0.02203868687349755</v>
       </c>
       <c r="J24" s="8" t="n">
         <v>961262</v>
@@ -1379,7 +1379,7 @@
         <v>90.5</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>0.1085966579317357</v>
+        <v>0.1085966579317358</v>
       </c>
       <c r="J26" s="8" t="n">
         <v>80262</v>
@@ -1395,34 +1395,34 @@
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>0.76</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.59</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>1.02</v>
+        <v>0.97</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.28</v>
+        <v>0.33</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>2.06</v>
+        <v>1.72</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>82.40000000000001</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.02000889385459848</v>
+        <v>0.02138366224399207</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>508427</v>
+        <v>511508</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>63225</v>
+        <v>63626</v>
       </c>
     </row>
     <row r="28">
@@ -1453,7 +1453,7 @@
         <v>87.2</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>4.147592651637327e-05</v>
+        <v>4.147592651637323e-05</v>
       </c>
       <c r="J28" s="8" t="n">
         <v>639823</v>
@@ -1490,7 +1490,7 @@
         <v>81.90000000000001</v>
       </c>
       <c r="I29" s="7" t="n">
-        <v>0.1779303397630421</v>
+        <v>0.177930339763042</v>
       </c>
       <c r="J29" s="8" t="n">
         <v>77198</v>
@@ -1595,7 +1595,7 @@
         <v>57</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>0.5607534123225346</v>
+        <v>0.5607534123225345</v>
       </c>
       <c r="J32" s="8" t="n">
         <v>87065</v>
@@ -1607,649 +1607,649 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>fermented_foods</t>
+          <t>yogurt</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>0.82</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0.65</v>
+        <v>0.73</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>1.04</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.36</v>
+        <v>0.57</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>1.91</v>
+        <v>1.2</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>90.8</v>
+        <v>58.7</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.5897124894853758</v>
+        <v>0.0321383112172301</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>190614</v>
+        <v>20962</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>42598</v>
+        <v>40377</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>vitamin_e</t>
+          <t>flax</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="C34" s="5" t="n">
-        <v>0.82</v>
+        <v>0.84</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>0.71</v>
+        <v>0.72</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="F34" s="5" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="G34" s="5" t="n">
-        <v>1.65</v>
-      </c>
+        <v>0.97</v>
+      </c>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="n"/>
       <c r="H34" s="6" t="n">
-        <v>85</v>
-      </c>
-      <c r="I34" s="7" t="n">
-        <v>0.2610709779752496</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I34" s="7" t="n"/>
       <c r="J34" s="8" t="n">
-        <v>558626</v>
+        <v>6369</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>157061</v>
+        <v>2999</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>yogurt</t>
+          <t>flaxseed</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>0.82</v>
+        <v>0.84</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="F35" s="5" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="G35" s="5" t="n">
-        <v>1.2</v>
-      </c>
+        <v>0.97</v>
+      </c>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
       <c r="H35" s="6" t="n">
-        <v>58.7</v>
-      </c>
-      <c r="I35" s="7" t="n">
-        <v>0.03213831121723015</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I35" s="7" t="n"/>
       <c r="J35" s="8" t="n">
-        <v>20962</v>
+        <v>6369</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>40377</v>
+        <v>2999</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>flax</t>
+          <t>vitamin_d</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>1</v>
+        <v>79</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>0.84</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>0.72</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
+        <v>0.88</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>1.1</v>
+      </c>
       <c r="H36" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="7" t="n"/>
+        <v>84.09999999999999</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>3.890419094017949e-09</v>
+      </c>
       <c r="J36" s="8" t="n">
-        <v>6369</v>
+        <v>1568223</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>2999</v>
+        <v>240235</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>flaxseed</t>
+          <t>melatonin</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="E37" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C37" s="5" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="D37" s="5" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="E37" s="5" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
+      <c r="F37" s="5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>1.31</v>
+      </c>
       <c r="H37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I37" s="7" t="n"/>
+        <v>42.3</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>0.9864318175325133</v>
+      </c>
       <c r="J37" s="8" t="n">
-        <v>6369</v>
+        <v>62422</v>
       </c>
       <c r="K37" s="8" t="n">
-        <v>2999</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>vitamin_d</t>
+          <t>vitamin_e</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>79</v>
+        <v>27</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="D38" s="5" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.75</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.88</v>
+        <v>0.97</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.65</v>
+        <v>0.47</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>1.1</v>
+        <v>1.56</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>84.09999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>3.89041909401795e-09</v>
+        <v>0.4053101026267988</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>1568223</v>
+        <v>588732</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>240235</v>
+        <v>160975</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>manganese</t>
+          <t>fermented_foods</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="D39" s="5" t="n">
-        <v>0.73</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
+        <v>1.07</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>1.87</v>
+      </c>
       <c r="H39" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" s="7" t="n"/>
+        <v>90.8</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>0.6093332948568931</v>
+      </c>
       <c r="J39" s="8" t="n">
-        <v>2939</v>
+        <v>218102</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>382</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>melatonin</t>
+          <t>green_tea</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="D40" s="5" t="n">
-        <v>0.73</v>
+        <v>0.77</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.55</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>1.31</v>
+        <v>1.4</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>42.3</v>
+        <v>85.7</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>0.9864318175325136</v>
+        <v>0.1921224493171251</v>
       </c>
       <c r="J40" s="8" t="n">
-        <v>62422</v>
+        <v>274406</v>
       </c>
       <c r="K40" s="8" t="n">
-        <v>3175</v>
+        <v>18211</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>green_tea</t>
+          <t>vitamin_a</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>0.89</v>
+        <v>0.9</v>
       </c>
       <c r="D41" s="5" t="n">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>1.02</v>
+        <v>1.08</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.44</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>1.4</v>
+        <v>1.84</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>85.7</v>
+        <v>86</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.192122449317125</v>
+        <v>0.4943075797793355</v>
       </c>
       <c r="J41" s="8" t="n">
-        <v>274406</v>
+        <v>551013</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>18211</v>
+        <v>143360</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>vitamin_a</t>
+          <t>calcium</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="D42" s="5" t="n">
-        <v>0.74</v>
+        <v>0.86</v>
       </c>
       <c r="E42" s="5" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G42" s="5" t="n">
         <v>1.08</v>
       </c>
-      <c r="F42" s="5" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="G42" s="5" t="n">
-        <v>1.84</v>
-      </c>
       <c r="H42" s="6" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>0.4943075797793356</v>
+        <v>0.0263926497392778</v>
       </c>
       <c r="J42" s="8" t="n">
-        <v>551013</v>
+        <v>894018</v>
       </c>
       <c r="K42" s="8" t="n">
-        <v>143360</v>
+        <v>76477</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>calcium</t>
+          <t>vitamin_c</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>0.91</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D43" s="5" t="n">
-        <v>0.86</v>
+        <v>0.82</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>0.96</v>
+        <v>1.06</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0.76</v>
+        <v>0.59</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>1.08</v>
+        <v>1.48</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>0.02639264973927776</v>
+        <v>0.5612991451474079</v>
       </c>
       <c r="J43" s="8" t="n">
-        <v>894018</v>
+        <v>512782</v>
       </c>
       <c r="K43" s="8" t="n">
-        <v>76477</v>
+        <v>35415</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>vitamin_c</t>
+          <t>selenium</t>
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="D44" s="5" t="n">
-        <v>0.82</v>
+        <v>0.88</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>1.06</v>
+        <v>1.03</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.59</v>
+        <v>0.74</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>1.48</v>
+        <v>1.22</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>83</v>
+        <v>58.4</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>0.5612991451474082</v>
+        <v>0.8524602198215493</v>
       </c>
       <c r="J44" s="8" t="n">
-        <v>512782</v>
+        <v>346098</v>
       </c>
       <c r="K44" s="8" t="n">
-        <v>35415</v>
+        <v>21359</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>selenium</t>
+          <t>caffeine</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>0.95</v>
+        <v>0.97</v>
       </c>
       <c r="D45" s="5" t="n">
-        <v>0.88</v>
+        <v>0.92</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.74</v>
+        <v>0.85</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>58.4</v>
+        <v>45.9</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>0.8524602198215492</v>
+        <v>0.4259906328747249</v>
       </c>
       <c r="J45" s="8" t="n">
-        <v>346098</v>
+        <v>872194</v>
       </c>
       <c r="K45" s="8" t="n">
-        <v>21359</v>
+        <v>38461</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>caffeine</t>
+          <t>bcaas</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>0.92</v>
+        <v>0.87</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>1.01</v>
+        <v>1.11</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.85</v>
+        <v>0.63</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>1.1</v>
+        <v>1.55</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>45.9</v>
+        <v>79.5</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0.4259906328747247</v>
+        <v>0.543858291819744</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>872194</v>
+        <v>224226</v>
       </c>
       <c r="K46" s="8" t="n">
-        <v>38461</v>
+        <v>14045</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>bcaas</t>
+          <t>dairy</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
-        <v>4</v>
+        <v>49</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>0.87</v>
+        <v>0.96</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>1.11</v>
+        <v>1.02</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.63</v>
+        <v>0.9</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1.55</v>
+        <v>1.09</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>79.5</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>0.5438582918197439</v>
+        <v>0.3148015453815154</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>224226</v>
+        <v>2900381</v>
       </c>
       <c r="K47" s="8" t="n">
-        <v>14045</v>
+        <v>201856</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>dairy</t>
+          <t>isoleucine</t>
         </is>
       </c>
       <c r="B48" s="4" t="n">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>0.99</v>
+        <v>1</v>
       </c>
       <c r="D48" s="5" t="n">
-        <v>0.96</v>
+        <v>0.87</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>1.02</v>
+        <v>1.14</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>0.9</v>
+        <v>0.57</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>1.09</v>
+        <v>1.74</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>84.09999999999999</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>0.314801545381515</v>
+        <v>0.9376775415524332</v>
       </c>
       <c r="J48" s="8" t="n">
-        <v>2900381</v>
+        <v>227916</v>
       </c>
       <c r="K48" s="8" t="n">
-        <v>201856</v>
+        <v>15865</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>isoleucine</t>
+          <t>leucine</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
         <v>4</v>
       </c>
       <c r="C49" s="5" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="D49" s="5" t="n">
-        <v>0.87</v>
+        <v>0.91</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>1.14</v>
+        <v>1.13</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>0.57</v>
+        <v>0.65</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>1.74</v>
+        <v>1.57</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>86.09999999999999</v>
+        <v>80.8</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>0.9376775415524331</v>
+        <v>0.5613202208181791</v>
       </c>
       <c r="J49" s="8" t="n">
-        <v>227916</v>
+        <v>225687</v>
       </c>
       <c r="K49" s="8" t="n">
-        <v>15865</v>
+        <v>15633</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>leucine</t>
+          <t>manganese</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C50" s="5" t="n">
         <v>1.01</v>
       </c>
       <c r="D50" s="5" t="n">
-        <v>0.91</v>
+        <v>0.73</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>1.13</v>
-      </c>
-      <c r="F50" s="5" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="G50" s="5" t="n">
-        <v>1.57</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="F50" s="5" t="n"/>
+      <c r="G50" s="5" t="n"/>
       <c r="H50" s="6" t="n">
-        <v>80.8</v>
-      </c>
-      <c r="I50" s="7" t="n">
-        <v>0.5613202208181793</v>
-      </c>
+        <v>94.40000000000001</v>
+      </c>
+      <c r="I50" s="7" t="n"/>
       <c r="J50" s="8" t="n">
-        <v>225687</v>
+        <v>225520</v>
       </c>
       <c r="K50" s="8" t="n">
-        <v>15633</v>
+        <v>29318</v>
       </c>
     </row>
     <row r="51">
@@ -2311,7 +2311,7 @@
         <v>90.5</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>0.8887019962528848</v>
+        <v>0.8887019962528852</v>
       </c>
       <c r="J52" s="8" t="n">
         <v>1885475</v>
@@ -2348,7 +2348,7 @@
         <v>91.09999999999999</v>
       </c>
       <c r="I53" s="7" t="n">
-        <v>0.8134382130434087</v>
+        <v>0.8134382130434088</v>
       </c>
       <c r="J53" s="8" t="n">
         <v>800654</v>
@@ -2360,199 +2360,205 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>quercetin</t>
+          <t>coenzyme_q10</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C54" s="5" t="n">
-        <v>1.05</v>
+        <v>1.03</v>
       </c>
       <c r="D54" s="5" t="n">
-        <v>0.83</v>
+        <v>0.71</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="F54" s="5" t="n"/>
-      <c r="G54" s="5" t="n"/>
+        <v>1.48</v>
+      </c>
+      <c r="F54" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G54" s="5" t="n">
+        <v>5.18</v>
+      </c>
       <c r="H54" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" s="7" t="n"/>
+        <v>80.59999999999999</v>
+      </c>
+      <c r="I54" s="7" t="n">
+        <v>0.7275832009506575</v>
+      </c>
       <c r="J54" s="8" t="n">
-        <v>90630</v>
+        <v>581814</v>
       </c>
       <c r="K54" s="8" t="n">
-        <v>710</v>
+        <v>75889</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>conjugated_linoleic_acid</t>
+          <t>quercetin</t>
         </is>
       </c>
       <c r="B55" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C55" s="5" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="D55" s="5" t="n">
-        <v>0.92</v>
+        <v>0.83</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="F55" s="5" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="G55" s="5" t="n">
-        <v>1.82</v>
-      </c>
+        <v>1.34</v>
+      </c>
+      <c r="F55" s="5" t="n"/>
+      <c r="G55" s="5" t="n"/>
       <c r="H55" s="6" t="n">
-        <v>62</v>
-      </c>
-      <c r="I55" s="7" t="n">
-        <v>0.4225544208553845</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I55" s="7" t="n"/>
       <c r="J55" s="8" t="n">
-        <v>380443</v>
+        <v>90630</v>
       </c>
       <c r="K55" s="8" t="n">
-        <v>17329</v>
+        <v>710</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>glucosamine</t>
+          <t>conjugated_linoleic_acid</t>
         </is>
       </c>
       <c r="B56" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C56" s="5" t="n">
         <v>1.06</v>
       </c>
       <c r="D56" s="5" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="F56" s="5" t="n"/>
-      <c r="G56" s="5" t="n"/>
+        <v>1.22</v>
+      </c>
+      <c r="F56" s="5" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G56" s="5" t="n">
+        <v>1.82</v>
+      </c>
       <c r="H56" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I56" s="7" t="n"/>
+        <v>62</v>
+      </c>
+      <c r="I56" s="7" t="n">
+        <v>0.4225544208553845</v>
+      </c>
       <c r="J56" s="8" t="n">
-        <v>41082</v>
+        <v>380443</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>5341</v>
+        <v>17329</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>grape</t>
+          <t>glucosamine</t>
         </is>
       </c>
       <c r="B57" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C57" s="5" t="n">
-        <v>1.08</v>
+        <v>1.06</v>
       </c>
       <c r="D57" s="5" t="n">
-        <v>0.36</v>
+        <v>0.93</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>3.21</v>
+        <v>1.21</v>
       </c>
       <c r="F57" s="5" t="n"/>
       <c r="G57" s="5" t="n"/>
       <c r="H57" s="6" t="n">
-        <v>89.3</v>
+        <v>0</v>
       </c>
       <c r="I57" s="7" t="n"/>
       <c r="J57" s="8" t="n">
-        <v>1816</v>
+        <v>41082</v>
       </c>
       <c r="K57" s="8" t="n">
-        <v>609</v>
+        <v>5341</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>magnesium</t>
+          <t>grape</t>
         </is>
       </c>
       <c r="B58" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C58" s="5" t="n">
         <v>1.08</v>
       </c>
       <c r="D58" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.36</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="F58" s="5" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="G58" s="5" t="n">
-        <v>1.78</v>
-      </c>
+        <v>3.21</v>
+      </c>
+      <c r="F58" s="5" t="n"/>
+      <c r="G58" s="5" t="n"/>
       <c r="H58" s="6" t="n">
-        <v>93</v>
-      </c>
-      <c r="I58" s="7" t="n">
-        <v>0.4685196145888207</v>
-      </c>
+        <v>89.3</v>
+      </c>
+      <c r="I58" s="7" t="n"/>
       <c r="J58" s="8" t="n">
-        <v>1239364</v>
+        <v>1816</v>
       </c>
       <c r="K58" s="8" t="n">
-        <v>266355</v>
+        <v>609</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>coenzyme_q10</t>
+          <t>magnesium</t>
         </is>
       </c>
       <c r="B59" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C59" s="5" t="n">
-        <v>1.1</v>
+        <v>1.08</v>
       </c>
       <c r="D59" s="5" t="n">
-        <v>0.36</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>3.34</v>
-      </c>
-      <c r="F59" s="5" t="n"/>
-      <c r="G59" s="5" t="n"/>
+        <v>1.25</v>
+      </c>
+      <c r="F59" s="5" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G59" s="5" t="n">
+        <v>1.78</v>
+      </c>
       <c r="H59" s="6" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="I59" s="7" t="n"/>
+        <v>93</v>
+      </c>
+      <c r="I59" s="7" t="n">
+        <v>0.4685196145888209</v>
+      </c>
       <c r="J59" s="8" t="n">
-        <v>3633</v>
+        <v>1239364</v>
       </c>
       <c r="K59" s="8" t="n">
-        <v>725</v>
+        <v>266355</v>
       </c>
     </row>
     <row r="60">
@@ -2645,7 +2651,7 @@
         <v>0</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>0.9877864190999566</v>
+        <v>0.987786419099957</v>
       </c>
       <c r="J62" s="8" t="n">
         <v>66508</v>
@@ -2719,7 +2725,7 @@
         <v>96</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>0.6073544042976849</v>
+        <v>0.6073544042976847</v>
       </c>
       <c r="J64" s="8" t="n">
         <v>119440</v>
@@ -2756,7 +2762,7 @@
         <v>80.59999999999999</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>0.1723925153093608</v>
+        <v>0.1723925153093609</v>
       </c>
       <c r="J65" s="8" t="n">
         <v>1376214</v>
@@ -2793,7 +2799,7 @@
         <v>86.90000000000001</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>0.9936223155021588</v>
+        <v>0.9936223155021582</v>
       </c>
       <c r="J66" s="8" t="n">
         <v>29311</v>
@@ -2830,7 +2836,7 @@
         <v>62.7</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>6.586804402476428e-05</v>
+        <v>6.586804402476424e-05</v>
       </c>
       <c r="J67" s="8" t="n">
         <v>249396</v>
@@ -2846,7 +2852,7 @@
         </is>
       </c>
       <c r="B68" s="4" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C68" s="5" t="n">
         <v>1.26</v>
@@ -2867,13 +2873,13 @@
         <v>90.09999999999999</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>8.11707600187357e-33</v>
+        <v>1.351025706854092e-32</v>
       </c>
       <c r="J68" s="8" t="n">
-        <v>16482295</v>
+        <v>16480697</v>
       </c>
       <c r="K68" s="8" t="n">
-        <v>1437638</v>
+        <v>1437588</v>
       </c>
     </row>
     <row r="69">
@@ -2935,7 +2941,7 @@
         <v>88.3</v>
       </c>
       <c r="I70" s="7" t="n">
-        <v>1.319761565701648e-10</v>
+        <v>1.319761565701661e-10</v>
       </c>
       <c r="J70" s="8" t="n">
         <v>1260095</v>
@@ -3003,7 +3009,7 @@
         <v>89</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>0.4612984675749361</v>
+        <v>0.4612984675749355</v>
       </c>
       <c r="J72" s="8" t="n">
         <v>65747</v>

</xml_diff>

<commit_message>
Exclude genetic proxy and Mendelian randomization studies
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -718,390 +718,390 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>mushrooms</t>
+          <t>vitamin_b6</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C8" s="5" t="n">
-        <v>0.59</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0.24</v>
+        <v>0.42</v>
       </c>
       <c r="E8" s="5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G8" s="5" t="n">
         <v>1.43</v>
       </c>
-      <c r="F8" s="5" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>16.99</v>
-      </c>
       <c r="H8" s="6" t="n">
-        <v>91.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.8882941697523908</v>
+        <v>0.006929997867264418</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>4428</v>
+        <v>92079</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>1957</v>
+        <v>8361</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>lutein</t>
+          <t>mushrooms</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>0.52</v>
+        <v>0.24</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.74</v>
+        <v>1.43</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>0.35</v>
+        <v>0.02</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>1.11</v>
+        <v>16.99</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>78.8</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.0008471154848143979</v>
+        <v>0.8882941697523908</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>1072840</v>
+        <v>4428</v>
       </c>
       <c r="K9" s="8" t="n">
-        <v>51083</v>
+        <v>1957</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b6</t>
+          <t>lutein</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>0.62</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>0.44</v>
+        <v>0.52</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.87</v>
+        <v>0.74</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.19</v>
+        <v>0.35</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>1.97</v>
+        <v>1.11</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>86.09999999999999</v>
+        <v>78.8</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>0.0003230528771021325</v>
+        <v>0.0008471154848143979</v>
       </c>
       <c r="J10" s="8" t="n">
-        <v>336188</v>
+        <v>1072840</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>40095</v>
+        <v>51083</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b12</t>
+          <t>antioxidants</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.66</v>
+        <v>0.65</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.48</v>
+        <v>0.53</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.91</v>
+        <v>0.8</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>0.23</v>
+        <v>0.3</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>1.9</v>
+        <v>1.4</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>87.3</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.02220092332067385</v>
+        <v>0.001739915084199531</v>
       </c>
       <c r="J11" s="8" t="n">
-        <v>88794</v>
+        <v>397778</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>11404</v>
+        <v>21055</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>omega-3_fatty_acids</t>
+          <t>vitamin_b12</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0.67</v>
+        <v>0.66</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.58</v>
+        <v>0.48</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.79</v>
+        <v>0.91</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.36</v>
+        <v>0.23</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>1.24</v>
+        <v>1.9</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>71.5</v>
+        <v>87.3</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>0.4514368397136518</v>
+        <v>0.02220092332067385</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>267959</v>
+        <v>88794</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>13978</v>
+        <v>11404</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>iodine</t>
+          <t>omega-3_fatty_acids</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>0.46</v>
+        <v>0.58</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
+        <v>0.79</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>1.24</v>
+      </c>
       <c r="H13" s="6" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="I13" s="7" t="n"/>
+        <v>71.5</v>
+      </c>
+      <c r="I13" s="7" t="n">
+        <v>0.4514368397136518</v>
+      </c>
       <c r="J13" s="8" t="n">
-        <v>3284</v>
+        <v>267959</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>1288</v>
+        <v>13978</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>n-acetylcysteine</t>
+          <t>iodine</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="E14" s="5" t="n">
         <v>1</v>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>0.73</v>
       </c>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
       <c r="H14" s="6" t="n">
-        <v>0</v>
+        <v>44.9</v>
       </c>
       <c r="I14" s="7" t="n"/>
       <c r="J14" s="8" t="n">
-        <v>91546</v>
+        <v>3284</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>11901</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>oats</t>
+          <t>lycopene</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0.3</v>
+        <v>0.57</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>1.27</v>
+      </c>
       <c r="H15" s="6" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="I15" s="7" t="n"/>
+        <v>80.2</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.04375419300824928</v>
+      </c>
       <c r="J15" s="8" t="n">
-        <v>28604</v>
+        <v>141249</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>1075</v>
+        <v>13606</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>garlic</t>
+          <t>n-acetylcysteine</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0.55</v>
+        <v>0.68</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>1.91</v>
-      </c>
+        <v>0.73</v>
+      </c>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
       <c r="H16" s="6" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="I16" s="7" t="n">
-        <v>0.1879066502188127</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I16" s="7" t="n"/>
       <c r="J16" s="8" t="n">
-        <v>243855</v>
+        <v>91546</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>1388</v>
+        <v>11901</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>lycopene</t>
+          <t>oats</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.83</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>1.27</v>
-      </c>
+        <v>1.65</v>
+      </c>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
       <c r="H17" s="6" t="n">
-        <v>87.40000000000001</v>
-      </c>
-      <c r="I17" s="7" t="n">
-        <v>0.001143089295674924</v>
-      </c>
+        <v>82.3</v>
+      </c>
+      <c r="I17" s="7" t="n"/>
       <c r="J17" s="8" t="n">
-        <v>370200</v>
+        <v>28604</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>136583</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>antioxidants</t>
+          <t>garlic</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>0.72</v>
+        <v>0.71</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.63</v>
+        <v>0.55</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.82</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.45</v>
+        <v>0.27</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1.14</v>
+        <v>1.91</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>85.2</v>
+        <v>44.2</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>0.0009624795570247788</v>
+        <v>0.1879066502188127</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>855680</v>
+        <v>243855</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>267009</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="19">
@@ -1607,75 +1607,81 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>yogurt</t>
+          <t>vitamin_d</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>5</v>
+        <v>76</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>0.82</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0.73</v>
+        <v>0.78</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.57</v>
+        <v>0.61</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>1.2</v>
+        <v>1.11</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>58.7</v>
+        <v>83.7</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.0321383112172301</v>
+        <v>3.144214406359958e-08</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>20962</v>
+        <v>1316249</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>40377</v>
+        <v>99950</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>flax</t>
+          <t>yogurt</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C34" s="5" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>1.2</v>
+      </c>
       <c r="H34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" s="7" t="n"/>
+        <v>58.7</v>
+      </c>
+      <c r="I34" s="7" t="n">
+        <v>0.0321383112172301</v>
+      </c>
       <c r="J34" s="8" t="n">
-        <v>6369</v>
+        <v>20962</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>2999</v>
+        <v>40377</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>flaxseed</t>
+          <t>flax</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
@@ -1706,38 +1712,32 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>vitamin_d</t>
+          <t>flaxseed</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>79</v>
+        <v>1</v>
       </c>
       <c r="C36" s="5" t="n">
         <v>0.84</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.72</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="F36" s="5" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="G36" s="5" t="n">
-        <v>1.1</v>
-      </c>
+        <v>0.97</v>
+      </c>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
       <c r="H36" s="6" t="n">
-        <v>84.09999999999999</v>
-      </c>
-      <c r="I36" s="7" t="n">
-        <v>3.890419094017949e-09</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I36" s="7" t="n"/>
       <c r="J36" s="8" t="n">
-        <v>1568223</v>
+        <v>6369</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>240235</v>
+        <v>2999</v>
       </c>
     </row>
     <row r="37">
@@ -1780,75 +1780,75 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>vitamin_e</t>
+          <t>fermented_foods</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>0.85</v>
+        <v>0.86</v>
       </c>
       <c r="D38" s="5" t="n">
-        <v>0.75</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>0.97</v>
+        <v>1.07</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.47</v>
+        <v>0.4</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>1.56</v>
+        <v>1.87</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>84.3</v>
+        <v>90.8</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>0.4053101026267988</v>
+        <v>0.6093332948568931</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>588732</v>
+        <v>218102</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>160975</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>fermented_foods</t>
+          <t>vitamin_e</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C39" s="5" t="n">
         <v>0.86</v>
       </c>
       <c r="D39" s="5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.71</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>1.07</v>
+        <v>1.03</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.4</v>
+        <v>0.37</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>1.87</v>
+        <v>1.97</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>90.8</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.6093332948568931</v>
+        <v>0.2357154134130869</v>
       </c>
       <c r="J39" s="8" t="n">
-        <v>218102</v>
+        <v>329245</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>46171</v>
+        <v>33624</v>
       </c>
     </row>
     <row r="40">
@@ -1895,7 +1895,7 @@
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C41" s="5" t="n">
         <v>0.9</v>
@@ -1904,25 +1904,25 @@
         <v>0.74</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>1.08</v>
+        <v>1.09</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>1.84</v>
+        <v>1.88</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.4943075797793355</v>
+        <v>0.5117296187637113</v>
       </c>
       <c r="J41" s="8" t="n">
-        <v>551013</v>
+        <v>322062</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>143360</v>
+        <v>20383</v>
       </c>
     </row>
     <row r="42">
@@ -2076,75 +2076,75 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>bcaas</t>
+          <t>dairy</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>0.87</v>
+        <v>0.92</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>1.11</v>
+        <v>1.03</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.63</v>
+        <v>0.75</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>1.55</v>
+        <v>1.27</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>79.5</v>
+        <v>84.3</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0.543858291819744</v>
+        <v>0.2402296603125188</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>224226</v>
+        <v>2055428</v>
       </c>
       <c r="K46" s="8" t="n">
-        <v>14045</v>
+        <v>92012</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>dairy</t>
+          <t>bcaas</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
-        <v>49</v>
+        <v>4</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>0.96</v>
+        <v>0.87</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>1.02</v>
+        <v>1.11</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.9</v>
+        <v>0.63</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1.09</v>
+        <v>1.55</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>84.09999999999999</v>
+        <v>79.5</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>0.3148015453815154</v>
+        <v>0.543858291819744</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>2900381</v>
+        <v>224226</v>
       </c>
       <c r="K47" s="8" t="n">
-        <v>201856</v>
+        <v>14045</v>
       </c>
     </row>
     <row r="48">
@@ -2224,38 +2224,44 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>manganese</t>
+          <t>magnesium</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C50" s="5" t="n">
         <v>1.01</v>
       </c>
       <c r="D50" s="5" t="n">
-        <v>0.73</v>
+        <v>0.8</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F50" s="5" t="n"/>
-      <c r="G50" s="5" t="n"/>
+        <v>1.29</v>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G50" s="5" t="n">
+        <v>15.95</v>
+      </c>
       <c r="H50" s="6" t="n">
-        <v>94.40000000000001</v>
-      </c>
-      <c r="I50" s="7" t="n"/>
+        <v>79.8</v>
+      </c>
+      <c r="I50" s="7" t="n">
+        <v>0.807342335170024</v>
+      </c>
       <c r="J50" s="8" t="n">
-        <v>225520</v>
+        <v>69780</v>
       </c>
       <c r="K50" s="8" t="n">
-        <v>29318</v>
+        <v>9994</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>vitamin_k</t>
+          <t>manganese</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
@@ -2265,22 +2271,22 @@
         <v>1.01</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>0.68</v>
+        <v>0.73</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="F51" s="5" t="n"/>
       <c r="G51" s="5" t="n"/>
       <c r="H51" s="6" t="n">
-        <v>91.8</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I51" s="7" t="n"/>
       <c r="J51" s="8" t="n">
-        <v>5048</v>
+        <v>225520</v>
       </c>
       <c r="K51" s="8" t="n">
-        <v>2592</v>
+        <v>29318</v>
       </c>
     </row>
     <row r="52">
@@ -2290,71 +2296,65 @@
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C52" s="5" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="D52" s="5" t="n">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0.74</v>
+        <v>0.66</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>1.4</v>
+        <v>1.53</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>90.5</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>0.8887019962528852</v>
+        <v>0.8949436838903885</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>1885475</v>
+        <v>1206930</v>
       </c>
       <c r="K52" s="8" t="n">
-        <v>231699</v>
+        <v>65930</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>carnitine</t>
+          <t>vitamin_k</t>
         </is>
       </c>
       <c r="B53" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C53" s="5" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="D53" s="5" t="n">
-        <v>0.82</v>
+        <v>0.68</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="F53" s="5" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="G53" s="5" t="n">
-        <v>2.45</v>
-      </c>
+        <v>1.5</v>
+      </c>
+      <c r="F53" s="5" t="n"/>
+      <c r="G53" s="5" t="n"/>
       <c r="H53" s="6" t="n">
-        <v>91.09999999999999</v>
-      </c>
-      <c r="I53" s="7" t="n">
-        <v>0.8134382130434088</v>
-      </c>
+        <v>91.8</v>
+      </c>
+      <c r="I53" s="7" t="n"/>
       <c r="J53" s="8" t="n">
-        <v>800654</v>
+        <v>5048</v>
       </c>
       <c r="K53" s="8" t="n">
-        <v>194212</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="54">
@@ -2397,11 +2397,11 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>quercetin</t>
+          <t>carnitine</t>
         </is>
       </c>
       <c r="B55" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C55" s="5" t="n">
         <v>1.05</v>
@@ -2410,155 +2410,155 @@
         <v>0.83</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="F55" s="5" t="n"/>
-      <c r="G55" s="5" t="n"/>
+        <v>1.35</v>
+      </c>
+      <c r="F55" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G55" s="5" t="n">
+        <v>19.83</v>
+      </c>
       <c r="H55" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I55" s="7" t="n"/>
+        <v>85.2</v>
+      </c>
+      <c r="I55" s="7" t="n">
+        <v>0.9420533281673373</v>
+      </c>
       <c r="J55" s="8" t="n">
-        <v>90630</v>
+        <v>5536</v>
       </c>
       <c r="K55" s="8" t="n">
-        <v>710</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>conjugated_linoleic_acid</t>
+          <t>quercetin</t>
         </is>
       </c>
       <c r="B56" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C56" s="5" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="D56" s="5" t="n">
-        <v>0.92</v>
+        <v>0.83</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>1.22</v>
-      </c>
-      <c r="F56" s="5" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="G56" s="5" t="n">
-        <v>1.82</v>
-      </c>
+        <v>1.34</v>
+      </c>
+      <c r="F56" s="5" t="n"/>
+      <c r="G56" s="5" t="n"/>
       <c r="H56" s="6" t="n">
-        <v>62</v>
-      </c>
-      <c r="I56" s="7" t="n">
-        <v>0.4225544208553845</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I56" s="7" t="n"/>
       <c r="J56" s="8" t="n">
-        <v>380443</v>
+        <v>90630</v>
       </c>
       <c r="K56" s="8" t="n">
-        <v>17329</v>
+        <v>710</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>glucosamine</t>
+          <t>conjugated_linoleic_acid</t>
         </is>
       </c>
       <c r="B57" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C57" s="5" t="n">
         <v>1.06</v>
       </c>
       <c r="D57" s="5" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>1.21</v>
-      </c>
-      <c r="F57" s="5" t="n"/>
-      <c r="G57" s="5" t="n"/>
+        <v>1.22</v>
+      </c>
+      <c r="F57" s="5" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G57" s="5" t="n">
+        <v>1.82</v>
+      </c>
       <c r="H57" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I57" s="7" t="n"/>
+        <v>62</v>
+      </c>
+      <c r="I57" s="7" t="n">
+        <v>0.4225544208553845</v>
+      </c>
       <c r="J57" s="8" t="n">
-        <v>41082</v>
+        <v>380443</v>
       </c>
       <c r="K57" s="8" t="n">
-        <v>5341</v>
+        <v>17329</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>grape</t>
+          <t>glucosamine</t>
         </is>
       </c>
       <c r="B58" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C58" s="5" t="n">
-        <v>1.08</v>
+        <v>1.06</v>
       </c>
       <c r="D58" s="5" t="n">
-        <v>0.36</v>
+        <v>0.93</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>3.21</v>
+        <v>1.21</v>
       </c>
       <c r="F58" s="5" t="n"/>
       <c r="G58" s="5" t="n"/>
       <c r="H58" s="6" t="n">
-        <v>89.3</v>
+        <v>0</v>
       </c>
       <c r="I58" s="7" t="n"/>
       <c r="J58" s="8" t="n">
-        <v>1816</v>
+        <v>41082</v>
       </c>
       <c r="K58" s="8" t="n">
-        <v>609</v>
+        <v>5341</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>magnesium</t>
+          <t>grape</t>
         </is>
       </c>
       <c r="B59" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C59" s="5" t="n">
         <v>1.08</v>
       </c>
       <c r="D59" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.36</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="F59" s="5" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="G59" s="5" t="n">
-        <v>1.78</v>
-      </c>
+        <v>3.21</v>
+      </c>
+      <c r="F59" s="5" t="n"/>
+      <c r="G59" s="5" t="n"/>
       <c r="H59" s="6" t="n">
-        <v>93</v>
-      </c>
-      <c r="I59" s="7" t="n">
-        <v>0.4685196145888209</v>
-      </c>
+        <v>89.3</v>
+      </c>
+      <c r="I59" s="7" t="n"/>
       <c r="J59" s="8" t="n">
-        <v>1239364</v>
+        <v>1816</v>
       </c>
       <c r="K59" s="8" t="n">
-        <v>266355</v>
+        <v>609</v>
       </c>
     </row>
     <row r="60">
@@ -2741,34 +2741,34 @@
         </is>
       </c>
       <c r="B65" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C65" s="5" t="n">
         <v>1.15</v>
       </c>
       <c r="D65" s="5" t="n">
-        <v>1.06</v>
+        <v>1.05</v>
       </c>
       <c r="E65" s="5" t="n">
         <v>1.25</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>1.58</v>
+        <v>1.6</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>80.59999999999999</v>
+        <v>81.2</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>0.1723925153093609</v>
+        <v>0.1931423553808721</v>
       </c>
       <c r="J65" s="8" t="n">
-        <v>1376214</v>
+        <v>1147263</v>
       </c>
       <c r="K65" s="8" t="n">
-        <v>221434</v>
+        <v>98457</v>
       </c>
     </row>
     <row r="66">
@@ -2811,248 +2811,248 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>dehydroepiandrosterone</t>
+          <t>alcohol</t>
         </is>
       </c>
       <c r="B67" s="4" t="n">
-        <v>15</v>
+        <v>206</v>
       </c>
       <c r="C67" s="5" t="n">
-        <v>1.25</v>
+        <v>1.26</v>
       </c>
       <c r="D67" s="5" t="n">
-        <v>1.15</v>
+        <v>1.24</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1.36</v>
+        <v>1.29</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>0.97</v>
+        <v>1.05</v>
       </c>
       <c r="G67" s="5" t="n">
-        <v>1.61</v>
+        <v>1.52</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>62.7</v>
+        <v>90.2</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>6.586804402476424e-05</v>
+        <v>1.054694151915899e-32</v>
       </c>
       <c r="J67" s="8" t="n">
-        <v>249396</v>
+        <v>16480697</v>
       </c>
       <c r="K67" s="8" t="n">
-        <v>127523</v>
+        <v>1314611</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>alcohol</t>
+          <t>red_meat</t>
         </is>
       </c>
       <c r="B68" s="4" t="n">
-        <v>207</v>
+        <v>35</v>
       </c>
       <c r="C68" s="5" t="n">
-        <v>1.26</v>
+        <v>1.27</v>
       </c>
       <c r="D68" s="5" t="n">
-        <v>1.23</v>
+        <v>1.2</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>1.29</v>
+        <v>1.34</v>
       </c>
       <c r="F68" s="5" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>1.52</v>
+        <v>1.61</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>90.09999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>1.351025706854092e-32</v>
+        <v>1.319761565701661e-10</v>
       </c>
       <c r="J68" s="8" t="n">
-        <v>16480697</v>
+        <v>1260095</v>
       </c>
       <c r="K68" s="8" t="n">
-        <v>1437588</v>
+        <v>70729</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>phosphorus</t>
+          <t>dehydroepiandrosterone</t>
         </is>
       </c>
       <c r="B69" s="4" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="C69" s="5" t="n">
-        <v>1.27</v>
+        <v>1.29</v>
       </c>
       <c r="D69" s="5" t="n">
-        <v>0.49</v>
+        <v>1.17</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="F69" s="5" t="n"/>
-      <c r="G69" s="5" t="n"/>
+        <v>1.41</v>
+      </c>
+      <c r="F69" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="5" t="n">
+        <v>1.66</v>
+      </c>
       <c r="H69" s="6" t="n">
-        <v>78.2</v>
-      </c>
-      <c r="I69" s="7" t="n"/>
+        <v>51.1</v>
+      </c>
+      <c r="I69" s="7" t="n">
+        <v>0.0009428631078015095</v>
+      </c>
       <c r="J69" s="8" t="n">
-        <v>229321</v>
+        <v>20445</v>
       </c>
       <c r="K69" s="8" t="n">
-        <v>123051</v>
+        <v>4546</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>red_meat</t>
+          <t>cannabidiol</t>
         </is>
       </c>
       <c r="B70" s="4" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="C70" s="5" t="n">
-        <v>1.27</v>
+        <v>1.4</v>
       </c>
       <c r="D70" s="5" t="n">
-        <v>1.2</v>
+        <v>1.39</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="F70" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G70" s="5" t="n">
-        <v>1.61</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="F70" s="5" t="n"/>
+      <c r="G70" s="5" t="n"/>
       <c r="H70" s="6" t="n">
-        <v>88.3</v>
-      </c>
-      <c r="I70" s="7" t="n">
-        <v>1.319761565701661e-10</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I70" s="7" t="n"/>
       <c r="J70" s="8" t="n">
-        <v>1260095</v>
+        <v>124896418350</v>
       </c>
       <c r="K70" s="8" t="n">
-        <v>70729</v>
+        <v>51623922</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>cannabidiol</t>
+          <t>copper</t>
         </is>
       </c>
       <c r="B71" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C71" s="5" t="n">
-        <v>1.4</v>
+        <v>1.66</v>
       </c>
       <c r="D71" s="5" t="n">
-        <v>1.39</v>
+        <v>1.07</v>
       </c>
       <c r="E71" s="5" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F71" s="5" t="n"/>
-      <c r="G71" s="5" t="n"/>
+        <v>2.56</v>
+      </c>
+      <c r="F71" s="5" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G71" s="5" t="n">
+        <v>7.5</v>
+      </c>
       <c r="H71" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I71" s="7" t="n"/>
+        <v>89</v>
+      </c>
+      <c r="I71" s="7" t="n">
+        <v>0.4612984675749355</v>
+      </c>
       <c r="J71" s="8" t="n">
-        <v>124896418350</v>
+        <v>65747</v>
       </c>
       <c r="K71" s="8" t="n">
-        <v>51623922</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>copper</t>
+          <t>omega-6_fatty_acids</t>
         </is>
       </c>
       <c r="B72" s="4" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C72" s="5" t="n">
-        <v>1.66</v>
+        <v>1.88</v>
       </c>
       <c r="D72" s="5" t="n">
-        <v>1.07</v>
+        <v>1.41</v>
       </c>
       <c r="E72" s="5" t="n">
-        <v>2.56</v>
+        <v>2.51</v>
       </c>
       <c r="F72" s="5" t="n">
-        <v>0.37</v>
+        <v>0.29</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>7.5</v>
+        <v>12.25</v>
       </c>
       <c r="H72" s="6" t="n">
-        <v>89</v>
+        <v>0</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>0.4612984675749355</v>
+        <v>0.3558547673635933</v>
       </c>
       <c r="J72" s="8" t="n">
-        <v>65747</v>
+        <v>3160</v>
       </c>
       <c r="K72" s="8" t="n">
-        <v>1930</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>omega-6_fatty_acids</t>
+          <t>phosphorus</t>
         </is>
       </c>
       <c r="B73" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C73" s="5" t="n">
-        <v>1.88</v>
+        <v>2.3</v>
       </c>
       <c r="D73" s="5" t="n">
-        <v>1.41</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="E73" s="5" t="n">
-        <v>2.51</v>
-      </c>
-      <c r="F73" s="5" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="G73" s="5" t="n">
-        <v>12.25</v>
-      </c>
+        <v>5.61</v>
+      </c>
+      <c r="F73" s="5" t="n"/>
+      <c r="G73" s="5" t="n"/>
       <c r="H73" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I73" s="7" t="n">
-        <v>0.3558547673635933</v>
-      </c>
+      <c r="I73" s="7" t="n"/>
       <c r="J73" s="8" t="n">
-        <v>3160</v>
+        <v>370</v>
       </c>
       <c r="K73" s="8" t="n">
-        <v>1518</v>
+        <v>74</v>
       </c>
     </row>
     <row r="74">

</xml_diff>

<commit_message>
Use cancer-specific risks for RR conversion
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -675,7 +675,7 @@
         <v>94.5</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>0.8351773861379138</v>
+        <v>0.8351773861379131</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>5809</v>
@@ -743,7 +743,7 @@
         <v>72.2</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.006929997867264418</v>
+        <v>0.006929997867264329</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>92079</v>
@@ -854,7 +854,7 @@
         <v>85.90000000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.001739915084199531</v>
+        <v>0.001739915084199511</v>
       </c>
       <c r="J11" s="8" t="n">
         <v>397778</v>
@@ -891,7 +891,7 @@
         <v>87.3</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>0.02220092332067385</v>
+        <v>0.02220092332067384</v>
       </c>
       <c r="J12" s="8" t="n">
         <v>88794</v>
@@ -928,7 +928,7 @@
         <v>71.5</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.4514368397136518</v>
+        <v>0.4514368397136499</v>
       </c>
       <c r="J13" s="8" t="n">
         <v>267959</v>
@@ -996,7 +996,7 @@
         <v>80.2</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>0.04375419300824928</v>
+        <v>0.04375419300824931</v>
       </c>
       <c r="J15" s="8" t="n">
         <v>141249</v>
@@ -1132,7 +1132,7 @@
         <v>82.90000000000001</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0.002411799505362664</v>
+        <v>0.002451592100662769</v>
       </c>
       <c r="J19" s="8" t="n">
         <v>1817569</v>
@@ -1200,7 +1200,7 @@
         <v>64.2</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3220215410089056</v>
+        <v>0.3220215410089058</v>
       </c>
       <c r="J21" s="8" t="n">
         <v>31455</v>
@@ -1237,7 +1237,7 @@
         <v>86.09999999999999</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>4.31581844897966e-05</v>
+        <v>4.315818448979668e-05</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>273560</v>
@@ -1416,7 +1416,7 @@
         <v>81.90000000000001</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.02138366224399207</v>
+        <v>0.02138366224399213</v>
       </c>
       <c r="J27" s="8" t="n">
         <v>511508</v>
@@ -1453,7 +1453,7 @@
         <v>87.2</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>4.147592651637323e-05</v>
+        <v>4.147592651637335e-05</v>
       </c>
       <c r="J28" s="8" t="n">
         <v>639823</v>
@@ -1555,10 +1555,10 @@
         <v>1.35</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>81.5</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.001821422591105356</v>
+        <v>0.001637387808489203</v>
       </c>
       <c r="J31" s="8" t="n">
         <v>1079347</v>
@@ -1595,7 +1595,7 @@
         <v>57</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>0.5607534123225345</v>
+        <v>0.5607534123225351</v>
       </c>
       <c r="J32" s="8" t="n">
         <v>87065</v>
@@ -1669,7 +1669,7 @@
         <v>58.7</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.0321383112172301</v>
+        <v>0.03213831121723015</v>
       </c>
       <c r="J34" s="8" t="n">
         <v>20962</v>
@@ -1805,7 +1805,7 @@
         <v>90.8</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>0.6093332948568931</v>
+        <v>0.6093332948568937</v>
       </c>
       <c r="J38" s="8" t="n">
         <v>218102</v>
@@ -1842,7 +1842,7 @@
         <v>86.09999999999999</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.2357154134130869</v>
+        <v>0.2376663782939103</v>
       </c>
       <c r="J39" s="8" t="n">
         <v>329245</v>
@@ -1916,7 +1916,7 @@
         <v>87</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.5117296187637113</v>
+        <v>0.5117296187637108</v>
       </c>
       <c r="J41" s="8" t="n">
         <v>322062</v>
@@ -1953,7 +1953,7 @@
         <v>81</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>0.0263926497392778</v>
+        <v>0.02639264973927816</v>
       </c>
       <c r="J42" s="8" t="n">
         <v>894018</v>
@@ -2064,7 +2064,7 @@
         <v>45.9</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>0.4259906328747249</v>
+        <v>0.4259906328747333</v>
       </c>
       <c r="J45" s="8" t="n">
         <v>872194</v>
@@ -2101,7 +2101,7 @@
         <v>84.3</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0.2402296603125188</v>
+        <v>0.2402296603125195</v>
       </c>
       <c r="J46" s="8" t="n">
         <v>2055428</v>
@@ -2138,7 +2138,7 @@
         <v>79.5</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>0.543858291819744</v>
+        <v>0.543858291819745</v>
       </c>
       <c r="J47" s="8" t="n">
         <v>224226</v>
@@ -2175,7 +2175,7 @@
         <v>86.09999999999999</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>0.9376775415524332</v>
+        <v>0.9376775415524354</v>
       </c>
       <c r="J48" s="8" t="n">
         <v>227916</v>
@@ -2212,7 +2212,7 @@
         <v>80.8</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>0.5613202208181791</v>
+        <v>0.5613202208181811</v>
       </c>
       <c r="J49" s="8" t="n">
         <v>225687</v>
@@ -2249,7 +2249,7 @@
         <v>79.8</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>0.807342335170024</v>
+        <v>0.8073423351700232</v>
       </c>
       <c r="J50" s="8" t="n">
         <v>69780</v>
@@ -2317,7 +2317,7 @@
         <v>91.09999999999999</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>0.8949436838903885</v>
+        <v>0.8949436838903891</v>
       </c>
       <c r="J52" s="8" t="n">
         <v>1206930</v>
@@ -2385,7 +2385,7 @@
         <v>80.59999999999999</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>0.7275832009506575</v>
+        <v>0.7275832009506582</v>
       </c>
       <c r="J54" s="8" t="n">
         <v>581814</v>
@@ -2422,7 +2422,7 @@
         <v>85.2</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>0.9420533281673373</v>
+        <v>0.9420533281673369</v>
       </c>
       <c r="J55" s="8" t="n">
         <v>5536</v>
@@ -2490,7 +2490,7 @@
         <v>62</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>0.4225544208553845</v>
+        <v>0.4225544208553847</v>
       </c>
       <c r="J57" s="8" t="n">
         <v>380443</v>
@@ -2725,7 +2725,7 @@
         <v>96</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>0.6073544042976847</v>
+        <v>0.6073544042976848</v>
       </c>
       <c r="J64" s="8" t="n">
         <v>119440</v>
@@ -2762,7 +2762,7 @@
         <v>81.2</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>0.1931423553808721</v>
+        <v>0.1931423553808725</v>
       </c>
       <c r="J65" s="8" t="n">
         <v>1147263</v>
@@ -2799,7 +2799,7 @@
         <v>86.90000000000001</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>0.9936223155021582</v>
+        <v>0.993622315502159</v>
       </c>
       <c r="J66" s="8" t="n">
         <v>29311</v>
@@ -2836,7 +2836,7 @@
         <v>90.2</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>1.054694151915899e-32</v>
+        <v>1.055446586763983e-32</v>
       </c>
       <c r="J67" s="8" t="n">
         <v>16480697</v>
@@ -2873,7 +2873,7 @@
         <v>88.3</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>1.319761565701661e-10</v>
+        <v>1.31976156570158e-10</v>
       </c>
       <c r="J68" s="8" t="n">
         <v>1260095</v>

</xml_diff>

<commit_message>
Remove duplicate vitamin E breast cancer study
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -1821,34 +1821,34 @@
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>0.86</v>
+        <v>0.82</v>
       </c>
       <c r="D39" s="5" t="n">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>1.03</v>
+        <v>0.97</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.37</v>
+        <v>0.38</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>1.97</v>
+        <v>1.77</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>86.09999999999999</v>
+        <v>84.5</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.2376663782939103</v>
+        <v>0.094160471030461</v>
       </c>
       <c r="J39" s="8" t="n">
-        <v>329245</v>
+        <v>328582</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>33624</v>
+        <v>33305</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
Exclude genetic-focus nutrition studies
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -588,100 +588,100 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>cesium</t>
+          <t>molybdenum</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C4" s="5" t="n">
-        <v>0.53</v>
+        <v>0.42</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>0.33</v>
+        <v>0.24</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
+        <v>0.76</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>586.39</v>
+      </c>
       <c r="H4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="7" t="n"/>
+        <v>95.09999999999999</v>
+      </c>
+      <c r="I4" s="7" t="n">
+        <v>0.5323616515032596</v>
+      </c>
       <c r="J4" s="8" t="n">
-        <v>486</v>
+        <v>4820</v>
       </c>
       <c r="K4" s="8" t="n">
-        <v>240</v>
+        <v>2330</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>potassium</t>
+          <t>cesium</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>0.55</v>
+        <v>0.53</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1.03</v>
+        <v>0.84</v>
       </c>
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="6" t="n">
-        <v>74.7</v>
+        <v>0</v>
       </c>
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="8" t="n">
-        <v>1370</v>
+        <v>486</v>
       </c>
       <c r="K5" s="8" t="n">
-        <v>587</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>molybdenum</t>
+          <t>potassium</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>6.78</v>
-      </c>
+        <v>1.03</v>
+      </c>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="6" t="n">
-        <v>94.5</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <v>0.8351773861379131</v>
-      </c>
+        <v>74.7</v>
+      </c>
+      <c r="I6" s="7" t="n"/>
       <c r="J6" s="8" t="n">
-        <v>5809</v>
+        <v>1370</v>
       </c>
       <c r="K6" s="8" t="n">
-        <v>2459</v>
+        <v>587</v>
       </c>
     </row>
     <row r="7">
@@ -743,7 +743,7 @@
         <v>72.2</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>0.006929997867264329</v>
+        <v>0.006929997867264313</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>92079</v>
@@ -780,7 +780,7 @@
         <v>91.90000000000001</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>0.8882941697523908</v>
+        <v>0.8882941697523911</v>
       </c>
       <c r="J9" s="8" t="n">
         <v>4428</v>
@@ -854,7 +854,7 @@
         <v>85.90000000000001</v>
       </c>
       <c r="I11" s="7" t="n">
-        <v>0.001739915084199511</v>
+        <v>0.001739915084199507</v>
       </c>
       <c r="J11" s="8" t="n">
         <v>397778</v>
@@ -866,656 +866,656 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b12</t>
+          <t>omega-3_fatty_acids</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.48</v>
+        <v>0.58</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.23</v>
+        <v>0.36</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>1.9</v>
+        <v>1.24</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>87.3</v>
+        <v>71.5</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>0.02220092332067384</v>
+        <v>0.45143683971365</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>88794</v>
+        <v>267959</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>11404</v>
+        <v>13978</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>omega-3_fatty_acids</t>
+          <t>lycopene</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.79</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="F13" s="5" t="n">
         <v>0.36</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>71.5</v>
+        <v>80.2</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.4514368397136499</v>
+        <v>0.04375419300824914</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>267959</v>
+        <v>141249</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>13978</v>
+        <v>13606</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>iodine</t>
+          <t>vitamin_b12</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>0.68</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>0.46</v>
+        <v>0.48</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
+        <v>0.95</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>2.04</v>
+      </c>
       <c r="H14" s="6" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="I14" s="7" t="n"/>
+        <v>88.40000000000001</v>
+      </c>
+      <c r="I14" s="7" t="n">
+        <v>0.03882289261966473</v>
+      </c>
       <c r="J14" s="8" t="n">
-        <v>3284</v>
+        <v>88394</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>1288</v>
+        <v>11275</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>lycopene</t>
+          <t>n-acetylcysteine</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C15" s="5" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D15" s="5" t="n">
         <v>0.68</v>
       </c>
-      <c r="D15" s="5" t="n">
-        <v>0.57</v>
-      </c>
       <c r="E15" s="5" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="F15" s="5" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="G15" s="5" t="n">
-        <v>1.27</v>
-      </c>
+        <v>0.73</v>
+      </c>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
       <c r="H15" s="6" t="n">
-        <v>80.2</v>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>0.04375419300824931</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I15" s="7" t="n"/>
       <c r="J15" s="8" t="n">
-        <v>141249</v>
+        <v>91546</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>13606</v>
+        <v>11901</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>n-acetylcysteine</t>
+          <t>oats</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="5" t="n">
         <v>0.7</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0.68</v>
+        <v>0.3</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.73</v>
+        <v>1.65</v>
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
       <c r="H16" s="6" t="n">
-        <v>0</v>
+        <v>82.3</v>
       </c>
       <c r="I16" s="7" t="n"/>
       <c r="J16" s="8" t="n">
-        <v>91546</v>
+        <v>28604</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>11901</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>oats</t>
+          <t>garlic</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>0.3</v>
+        <v>0.55</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>1.91</v>
+      </c>
       <c r="H17" s="6" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="I17" s="7" t="n"/>
+        <v>44.2</v>
+      </c>
+      <c r="I17" s="7" t="n">
+        <v>0.1879066502188127</v>
+      </c>
       <c r="J17" s="8" t="n">
-        <v>28604</v>
+        <v>243855</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>1075</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>garlic</t>
+          <t>beta-carotene</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.55</v>
+        <v>0.66</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.8</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.27</v>
+        <v>0.45</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>1.91</v>
+        <v>1.19</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>44.2</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>0.1879066502188127</v>
+        <v>0.002451592100662776</v>
       </c>
       <c r="J18" s="8" t="n">
-        <v>243855</v>
+        <v>1817569</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>1388</v>
+        <v>128023</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>beta-carotene</t>
+          <t>mineral_supplements</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>0.73</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>0.66</v>
+        <v>0.43</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>1.19</v>
-      </c>
+        <v>1.17</v>
+      </c>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
       <c r="H19" s="6" t="n">
-        <v>82.90000000000001</v>
-      </c>
-      <c r="I19" s="7" t="n">
-        <v>0.002451592100662769</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I19" s="7" t="n"/>
       <c r="J19" s="8" t="n">
-        <v>1817569</v>
+        <v>836</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>128023</v>
+        <v>312</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>mineral_supplements</t>
+          <t>black_cohosh</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.43</v>
+        <v>0.6</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
+        <v>0.92</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>7.42</v>
+      </c>
       <c r="H20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="7" t="n"/>
+        <v>64.2</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>0.322021541008906</v>
+      </c>
       <c r="J20" s="8" t="n">
-        <v>836</v>
+        <v>31455</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>312</v>
+        <v>5515</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>black_cohosh</t>
+          <t>legumes</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>0.74</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>0.6</v>
+        <v>0.65</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="G21" s="5" t="n">
-        <v>7.42</v>
+        <v>1.22</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>64.2</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>0.3220215410089058</v>
+        <v>4.315818448979673e-05</v>
       </c>
       <c r="J21" s="8" t="n">
-        <v>31455</v>
+        <v>273560</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>5515</v>
+        <v>15479</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>legumes</t>
+          <t>olive</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.45</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>1.22</v>
+        <v>1.24</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>86.09999999999999</v>
+        <v>84.8</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>4.315818448979668e-05</v>
+        <v>0.005850985088450088</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>273560</v>
+        <v>249237</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>15479</v>
+        <v>17161</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>olive</t>
+          <t>soy</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>0.75</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.45</v>
+        <v>0.32</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>1.24</v>
+        <v>1.75</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>84.8</v>
+        <v>90.8</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.005850985088450085</v>
+        <v>0.02203868687349753</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>249237</v>
+        <v>961262</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>17161</v>
+        <v>34226</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>soy</t>
+          <t>vitamin_b1</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>0.75</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>0.65</v>
+        <v>0.61</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="F24" s="5" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>1.75</v>
-      </c>
+        <v>0.93</v>
+      </c>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
       <c r="H24" s="6" t="n">
-        <v>90.8</v>
-      </c>
-      <c r="I24" s="7" t="n">
-        <v>0.02203868687349755</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I24" s="7" t="n"/>
       <c r="J24" s="8" t="n">
-        <v>961262</v>
+        <v>38639</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>34226</v>
+        <v>853</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b1</t>
+          <t>choline</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>0.61</v>
+        <v>0.52</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
+        <v>1.11</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>4.41</v>
+      </c>
       <c r="H25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I25" s="7" t="n"/>
+        <v>90.5</v>
+      </c>
+      <c r="I25" s="7" t="n">
+        <v>0.1085966579317357</v>
+      </c>
       <c r="J25" s="8" t="n">
-        <v>38639</v>
+        <v>80262</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>853</v>
+        <v>6805</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>choline</t>
+          <t>fish_oil</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>0.76</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>0.52</v>
+        <v>0.59</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>1.11</v>
+        <v>0.97</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.13</v>
+        <v>0.33</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>4.41</v>
+        <v>1.72</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>90.5</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>0.1085966579317358</v>
+        <v>0.02138366224399213</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>80262</v>
+        <v>511508</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>6805</v>
+        <v>63626</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>fish_oil</t>
+          <t>mediterranean_diet</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>0.76</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>0.59</v>
+        <v>0.7</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>0.97</v>
+        <v>0.83</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.33</v>
+        <v>0.54</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>1.72</v>
+        <v>1.08</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>81.90000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>0.02138366224399213</v>
+        <v>4.147592651637327e-05</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>511508</v>
+        <v>639823</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>63626</v>
+        <v>40922</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>mediterranean_diet</t>
+          <t>betaine</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>0.7</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>0.83</v>
+        <v>1.07</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.54</v>
+        <v>0.02</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>1.08</v>
+        <v>37.25</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>87.2</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>4.147592651637335e-05</v>
+        <v>0.1779303397630421</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>639823</v>
+        <v>77198</v>
       </c>
       <c r="K28" s="8" t="n">
-        <v>40922</v>
+        <v>5297</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>betaine</t>
+          <t>cod_liver_oil</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.68</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="F29" s="5" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="G29" s="5" t="n">
-        <v>37.25</v>
-      </c>
+        <v>0.9</v>
+      </c>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
       <c r="H29" s="6" t="n">
-        <v>81.90000000000001</v>
-      </c>
-      <c r="I29" s="7" t="n">
-        <v>0.177930339763042</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I29" s="7" t="n"/>
       <c r="J29" s="8" t="n">
-        <v>77198</v>
+        <v>4001</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>5297</v>
+        <v>1731</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>cod_liver_oil</t>
+          <t>iodine</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>0.78</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>0.68</v>
+        <v>0.6</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.9</v>
+        <v>0.99</v>
       </c>
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="5" t="n"/>
@@ -1524,10 +1524,10 @@
       </c>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="8" t="n">
-        <v>4001</v>
+        <v>2295</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>1731</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="31">
@@ -1537,34 +1537,34 @@
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="F31" s="5" t="n">
         <v>0.47</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="H31" s="6" t="n">
         <v>81.59999999999999</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>0.001637387808489203</v>
+        <v>0.002768602416666183</v>
       </c>
       <c r="J31" s="8" t="n">
-        <v>1079347</v>
+        <v>1078947</v>
       </c>
       <c r="K31" s="8" t="n">
-        <v>52296</v>
+        <v>52167</v>
       </c>
     </row>
     <row r="32">
@@ -1595,7 +1595,7 @@
         <v>57</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>0.5607534123225351</v>
+        <v>0.5607534123225348</v>
       </c>
       <c r="J32" s="8" t="n">
         <v>87065</v>
@@ -1611,13 +1611,13 @@
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>0.82</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="E33" s="5" t="n">
         <v>0.86</v>
@@ -1629,90 +1629,96 @@
         <v>1.11</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>83.7</v>
+        <v>83.8</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>3.144214406359958e-08</v>
+        <v>5.261486437358412e-08</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>1316249</v>
+        <v>1315839</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>99950</v>
+        <v>99816</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>yogurt</t>
+          <t>vitamin_e</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>0.82</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>0.73</v>
+        <v>0.68</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.57</v>
+        <v>0.38</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>1.2</v>
+        <v>1.77</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>58.7</v>
+        <v>84.5</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.03213831121723015</v>
+        <v>0.094160471030461</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>20962</v>
+        <v>328582</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>40377</v>
+        <v>33305</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>flax</t>
+          <t>yogurt</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C35" s="5" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>1.2</v>
+      </c>
       <c r="H35" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="7" t="n"/>
+        <v>58.7</v>
+      </c>
+      <c r="I35" s="7" t="n">
+        <v>0.03213831121723015</v>
+      </c>
       <c r="J35" s="8" t="n">
-        <v>6369</v>
+        <v>20962</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>2999</v>
+        <v>40377</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>flaxseed</t>
+          <t>flax</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
@@ -1743,112 +1749,106 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>melatonin</t>
+          <t>flaxseed</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C37" s="5" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="D37" s="5" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="5" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="G37" s="5" t="n">
-        <v>1.31</v>
-      </c>
+        <v>0.97</v>
+      </c>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
       <c r="H37" s="6" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="I37" s="7" t="n">
-        <v>0.9864318175325133</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I37" s="7" t="n"/>
       <c r="J37" s="8" t="n">
-        <v>62422</v>
+        <v>6369</v>
       </c>
       <c r="K37" s="8" t="n">
-        <v>3175</v>
+        <v>2999</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>fermented_foods</t>
+          <t>melatonin</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="D38" s="5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.73</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>1.07</v>
+        <v>1</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>1.87</v>
+        <v>1.31</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>90.8</v>
+        <v>42.3</v>
       </c>
       <c r="I38" s="7" t="n">
-        <v>0.6093332948568937</v>
+        <v>0.9864318175325136</v>
       </c>
       <c r="J38" s="8" t="n">
-        <v>218102</v>
+        <v>62422</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>46171</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>vitamin_e</t>
+          <t>fermented_foods</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="D39" s="5" t="n">
-        <v>0.68</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>0.97</v>
+        <v>1.07</v>
       </c>
       <c r="F39" s="5" t="n">
-        <v>0.38</v>
+        <v>0.4</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>1.77</v>
+        <v>1.87</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>84.5</v>
+        <v>90.8</v>
       </c>
       <c r="I39" s="7" t="n">
-        <v>0.094160471030461</v>
+        <v>0.6093332948568936</v>
       </c>
       <c r="J39" s="8" t="n">
-        <v>328582</v>
+        <v>218102</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>33305</v>
+        <v>46171</v>
       </c>
     </row>
     <row r="40">
@@ -1879,7 +1879,7 @@
         <v>85.7</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>0.1921224493171251</v>
+        <v>0.192122449317125</v>
       </c>
       <c r="J40" s="8" t="n">
         <v>274406</v>
@@ -1916,7 +1916,7 @@
         <v>87</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.5117296187637108</v>
+        <v>0.5117296187637109</v>
       </c>
       <c r="J41" s="8" t="n">
         <v>322062</v>
@@ -1953,7 +1953,7 @@
         <v>81</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>0.02639264973927816</v>
+        <v>0.02639264973927821</v>
       </c>
       <c r="J42" s="8" t="n">
         <v>894018</v>
@@ -1990,7 +1990,7 @@
         <v>83</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>0.5612991451474079</v>
+        <v>0.5612991451474082</v>
       </c>
       <c r="J43" s="8" t="n">
         <v>512782</v>
@@ -2027,7 +2027,7 @@
         <v>58.4</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>0.8524602198215493</v>
+        <v>0.8524602198215492</v>
       </c>
       <c r="J44" s="8" t="n">
         <v>346098</v>
@@ -2064,7 +2064,7 @@
         <v>45.9</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>0.4259906328747333</v>
+        <v>0.4259906328747331</v>
       </c>
       <c r="J45" s="8" t="n">
         <v>872194</v>
@@ -2101,7 +2101,7 @@
         <v>84.3</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0.2402296603125195</v>
+        <v>0.240229660312519</v>
       </c>
       <c r="J46" s="8" t="n">
         <v>2055428</v>
@@ -2117,7 +2117,7 @@
         </is>
       </c>
       <c r="B47" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C47" s="5" t="n">
         <v>0.98</v>
@@ -2126,25 +2126,25 @@
         <v>0.87</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>1.11</v>
+        <v>1.1</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.63</v>
+        <v>0.25</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>1.55</v>
+        <v>3.8</v>
       </c>
       <c r="H47" s="6" t="n">
-        <v>79.5</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>0.543858291819745</v>
+        <v>0.2941582730123437</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>224226</v>
+        <v>223922</v>
       </c>
       <c r="K47" s="8" t="n">
-        <v>14045</v>
+        <v>13868</v>
       </c>
     </row>
     <row r="48">
@@ -2175,7 +2175,7 @@
         <v>86.09999999999999</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>0.9376775415524354</v>
+        <v>0.9376775415524352</v>
       </c>
       <c r="J48" s="8" t="n">
         <v>227916</v>
@@ -2212,7 +2212,7 @@
         <v>80.8</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>0.5613202208181811</v>
+        <v>0.5613202208181812</v>
       </c>
       <c r="J49" s="8" t="n">
         <v>225687</v>
@@ -2249,7 +2249,7 @@
         <v>79.8</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>0.8073423351700232</v>
+        <v>0.8073423351700231</v>
       </c>
       <c r="J50" s="8" t="n">
         <v>69780</v>
@@ -2317,7 +2317,7 @@
         <v>91.09999999999999</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>0.8949436838903891</v>
+        <v>0.894943683890389</v>
       </c>
       <c r="J52" s="8" t="n">
         <v>1206930</v>
@@ -2385,7 +2385,7 @@
         <v>80.59999999999999</v>
       </c>
       <c r="I54" s="7" t="n">
-        <v>0.7275832009506582</v>
+        <v>0.727583200950658</v>
       </c>
       <c r="J54" s="8" t="n">
         <v>581814</v>
@@ -2422,7 +2422,7 @@
         <v>85.2</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>0.9420533281673369</v>
+        <v>0.9420533281673368</v>
       </c>
       <c r="J55" s="8" t="n">
         <v>5536</v>
@@ -2490,7 +2490,7 @@
         <v>62</v>
       </c>
       <c r="I57" s="7" t="n">
-        <v>0.4225544208553847</v>
+        <v>0.4225544208553849</v>
       </c>
       <c r="J57" s="8" t="n">
         <v>380443</v>
@@ -2651,7 +2651,7 @@
         <v>0</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>0.987786419099957</v>
+        <v>0.9877864190999566</v>
       </c>
       <c r="J62" s="8" t="n">
         <v>66508</v>
@@ -2725,7 +2725,7 @@
         <v>96</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>0.6073544042976848</v>
+        <v>0.6073544042976849</v>
       </c>
       <c r="J64" s="8" t="n">
         <v>119440</v>
@@ -2799,7 +2799,7 @@
         <v>86.90000000000001</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>0.993622315502159</v>
+        <v>0.9936223155021582</v>
       </c>
       <c r="J66" s="8" t="n">
         <v>29311</v>
@@ -2815,10 +2815,10 @@
         </is>
       </c>
       <c r="B67" s="4" t="n">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C67" s="5" t="n">
-        <v>1.26</v>
+        <v>1.27</v>
       </c>
       <c r="D67" s="5" t="n">
         <v>1.24</v>
@@ -2830,19 +2830,19 @@
         <v>1.05</v>
       </c>
       <c r="G67" s="5" t="n">
-        <v>1.52</v>
+        <v>1.53</v>
       </c>
       <c r="H67" s="6" t="n">
         <v>90.2</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>1.055446586763983e-32</v>
+        <v>7.90723755922392e-33</v>
       </c>
       <c r="J67" s="8" t="n">
-        <v>16480697</v>
+        <v>16471419</v>
       </c>
       <c r="K67" s="8" t="n">
-        <v>1314611</v>
+        <v>1313337</v>
       </c>
     </row>
     <row r="68">
@@ -2873,7 +2873,7 @@
         <v>88.3</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>1.31976156570158e-10</v>
+        <v>1.319761565701576e-10</v>
       </c>
       <c r="J68" s="8" t="n">
         <v>1260095</v>
@@ -2910,7 +2910,7 @@
         <v>51.1</v>
       </c>
       <c r="I69" s="7" t="n">
-        <v>0.0009428631078015095</v>
+        <v>0.0009428631078015041</v>
       </c>
       <c r="J69" s="8" t="n">
         <v>20445</v>
@@ -2978,7 +2978,7 @@
         <v>89</v>
       </c>
       <c r="I71" s="7" t="n">
-        <v>0.4612984675749355</v>
+        <v>0.4612984675749361</v>
       </c>
       <c r="J71" s="8" t="n">
         <v>65747</v>

</xml_diff>

<commit_message>
Sync evidence fixes and regenerate multilingual figures
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -792,730 +792,724 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>lutein</t>
+          <t>black_cohosh</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>0.52</v>
+        <v>0.34</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>1.11</v>
-      </c>
+        <v>1.07</v>
+      </c>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="6" t="n">
-        <v>78.8</v>
-      </c>
-      <c r="I10" s="7" t="n">
-        <v>0.0008471154848143979</v>
-      </c>
+        <v>76.40000000000001</v>
+      </c>
+      <c r="I10" s="7" t="n"/>
       <c r="J10" s="8" t="n">
-        <v>1072840</v>
+        <v>12594</v>
       </c>
       <c r="K10" s="8" t="n">
-        <v>51083</v>
+        <v>4413</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>antioxidants</t>
+          <t>grape</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C11" s="5" t="n">
-        <v>0.65</v>
+        <v>0.62</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>0.53</v>
+        <v>0.38</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>1.4</v>
-      </c>
+        <v>0.96</v>
+      </c>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
       <c r="H11" s="6" t="n">
-        <v>85.90000000000001</v>
-      </c>
-      <c r="I11" s="7" t="n">
-        <v>0.001739915084199507</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I11" s="7" t="n"/>
       <c r="J11" s="8" t="n">
-        <v>397778</v>
+        <v>1067</v>
       </c>
       <c r="K11" s="8" t="n">
-        <v>21055</v>
+        <v>359</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>omega-3_fatty_acids</t>
+          <t>lutein</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>0.67</v>
+        <v>0.62</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>0.58</v>
+        <v>0.52</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>0.79</v>
+        <v>0.74</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.36</v>
+        <v>0.35</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>1.24</v>
+        <v>1.11</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>71.5</v>
+        <v>78.8</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>0.45143683971365</v>
+        <v>0.0008471154848143979</v>
       </c>
       <c r="J12" s="8" t="n">
-        <v>267959</v>
+        <v>1072840</v>
       </c>
       <c r="K12" s="8" t="n">
-        <v>13978</v>
+        <v>51083</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>lycopene</t>
+          <t>antioxidants</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" s="5" t="n">
-        <v>0.68</v>
+        <v>0.65</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>0.57</v>
+        <v>0.53</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.36</v>
+        <v>0.3</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>1.27</v>
+        <v>1.4</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>80.2</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="I13" s="7" t="n">
-        <v>0.04375419300824914</v>
+        <v>0.001739915084199507</v>
       </c>
       <c r="J13" s="8" t="n">
-        <v>141249</v>
+        <v>397778</v>
       </c>
       <c r="K13" s="8" t="n">
-        <v>13606</v>
+        <v>21055</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b12</t>
+          <t>omega-3_fatty_acids</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>0.68</v>
+        <v>0.65</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>0.48</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.95</v>
+        <v>0.76</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0.22</v>
+        <v>0.36</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>2.04</v>
+        <v>1.17</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>88.40000000000001</v>
+        <v>68</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>0.03882289261966473</v>
+        <v>0.5929735955651908</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>88394</v>
+        <v>242088</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>11275</v>
+        <v>10615</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>n-acetylcysteine</t>
+          <t>lycopene</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>0.68</v>
+        <v>0.57</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>1.27</v>
+      </c>
       <c r="H15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="7" t="n"/>
+        <v>80.2</v>
+      </c>
+      <c r="I15" s="7" t="n">
+        <v>0.04375419300824914</v>
+      </c>
       <c r="J15" s="8" t="n">
-        <v>91546</v>
+        <v>141249</v>
       </c>
       <c r="K15" s="8" t="n">
-        <v>11901</v>
+        <v>13606</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>oats</t>
+          <t>vitamin_b12</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>0.3</v>
+        <v>0.48</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
+        <v>0.95</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>2.04</v>
+      </c>
       <c r="H16" s="6" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="I16" s="7" t="n"/>
+        <v>88.40000000000001</v>
+      </c>
+      <c r="I16" s="7" t="n">
+        <v>0.03882289261966473</v>
+      </c>
       <c r="J16" s="8" t="n">
-        <v>28604</v>
+        <v>88394</v>
       </c>
       <c r="K16" s="8" t="n">
-        <v>1075</v>
+        <v>11275</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>garlic</t>
+          <t>n-acetylcysteine</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>0.71</v>
+        <v>0.7</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>0.55</v>
+        <v>0.68</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="F17" s="5" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="G17" s="5" t="n">
-        <v>1.91</v>
-      </c>
+        <v>0.73</v>
+      </c>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
       <c r="H17" s="6" t="n">
-        <v>44.2</v>
-      </c>
-      <c r="I17" s="7" t="n">
-        <v>0.1879066502188127</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I17" s="7" t="n"/>
       <c r="J17" s="8" t="n">
-        <v>243855</v>
+        <v>91546</v>
       </c>
       <c r="K17" s="8" t="n">
-        <v>1388</v>
+        <v>11901</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>beta-carotene</t>
+          <t>oats</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>0.73</v>
+        <v>0.7</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>0.66</v>
+        <v>0.3</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F18" s="5" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>1.19</v>
-      </c>
+        <v>1.65</v>
+      </c>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
       <c r="H18" s="6" t="n">
-        <v>82.90000000000001</v>
-      </c>
-      <c r="I18" s="7" t="n">
-        <v>0.002451592100662776</v>
-      </c>
+        <v>82.3</v>
+      </c>
+      <c r="I18" s="7" t="n"/>
       <c r="J18" s="8" t="n">
-        <v>1817569</v>
+        <v>28604</v>
       </c>
       <c r="K18" s="8" t="n">
-        <v>128023</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>mineral_supplements</t>
+          <t>garlic</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>0.43</v>
+        <v>0.55</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>1.17</v>
-      </c>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>1.91</v>
+      </c>
       <c r="H19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="7" t="n"/>
+        <v>44.2</v>
+      </c>
+      <c r="I19" s="7" t="n">
+        <v>0.1879066502188127</v>
+      </c>
       <c r="J19" s="8" t="n">
-        <v>836</v>
+        <v>243855</v>
       </c>
       <c r="K19" s="8" t="n">
-        <v>312</v>
+        <v>1388</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>black_cohosh</t>
+          <t>beta-carotene</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>3</v>
+        <v>39</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.45</v>
       </c>
       <c r="G20" s="5" t="n">
-        <v>7.42</v>
+        <v>1.19</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>64.2</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>0.322021541008906</v>
+        <v>0.002451592100662776</v>
       </c>
       <c r="J20" s="8" t="n">
-        <v>31455</v>
+        <v>1817569</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>5515</v>
+        <v>128023</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>legumes</t>
+          <t>mineral_supplements</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C21" s="5" t="n">
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>0.65</v>
+        <v>0.43</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F21" s="5" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>1.22</v>
-      </c>
+        <v>1.17</v>
+      </c>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
       <c r="H21" s="6" t="n">
-        <v>86.09999999999999</v>
-      </c>
-      <c r="I21" s="7" t="n">
-        <v>4.315818448979673e-05</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I21" s="7" t="n"/>
       <c r="J21" s="8" t="n">
-        <v>273560</v>
+        <v>836</v>
       </c>
       <c r="K21" s="8" t="n">
-        <v>15479</v>
+        <v>312</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>olive</t>
+          <t>legumes</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>0.64</v>
+        <v>0.65</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.87</v>
+        <v>0.85</v>
       </c>
       <c r="F22" s="5" t="n">
         <v>0.45</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>1.24</v>
+        <v>1.22</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>84.8</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>0.005850985088450088</v>
+        <v>4.315818448979673e-05</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>249237</v>
+        <v>273560</v>
       </c>
       <c r="K22" s="8" t="n">
-        <v>17161</v>
+        <v>15479</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>soy</t>
+          <t>olive</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>0.75</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.86</v>
+        <v>0.87</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.32</v>
+        <v>0.45</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>1.75</v>
+        <v>1.24</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>90.8</v>
+        <v>84.8</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>0.02203868687349753</v>
+        <v>0.005850985088450088</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>961262</v>
+        <v>249237</v>
       </c>
       <c r="K23" s="8" t="n">
-        <v>34226</v>
+        <v>17161</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>vitamin_b1</t>
+          <t>soy</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>0.75</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>0.61</v>
+        <v>0.65</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
+        <v>0.86</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>1.75</v>
+      </c>
       <c r="H24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" s="7" t="n"/>
+        <v>90.8</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>0.02203868687349753</v>
+      </c>
       <c r="J24" s="8" t="n">
-        <v>38639</v>
+        <v>961262</v>
       </c>
       <c r="K24" s="8" t="n">
-        <v>853</v>
+        <v>34226</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>choline</t>
+          <t>vitamin_b1</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C25" s="5" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>0.52</v>
+        <v>0.61</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>1.11</v>
-      </c>
-      <c r="F25" s="5" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>4.41</v>
-      </c>
+        <v>0.93</v>
+      </c>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
       <c r="H25" s="6" t="n">
-        <v>90.5</v>
-      </c>
-      <c r="I25" s="7" t="n">
-        <v>0.1085966579317357</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I25" s="7" t="n"/>
       <c r="J25" s="8" t="n">
-        <v>80262</v>
+        <v>38639</v>
       </c>
       <c r="K25" s="8" t="n">
-        <v>6805</v>
+        <v>853</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>fish_oil</t>
+          <t>choline</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>0.76</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>0.59</v>
+        <v>0.52</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>0.97</v>
+        <v>1.11</v>
       </c>
       <c r="F26" s="5" t="n">
-        <v>0.33</v>
+        <v>0.13</v>
       </c>
       <c r="G26" s="5" t="n">
-        <v>1.72</v>
+        <v>4.41</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>81.90000000000001</v>
+        <v>90.5</v>
       </c>
       <c r="I26" s="7" t="n">
-        <v>0.02138366224399213</v>
+        <v>0.1085966579317357</v>
       </c>
       <c r="J26" s="8" t="n">
-        <v>511508</v>
+        <v>80262</v>
       </c>
       <c r="K26" s="8" t="n">
-        <v>63626</v>
+        <v>6805</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>mediterranean_diet</t>
+          <t>fish_oil</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>0.76</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>0.7</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>0.83</v>
+        <v>1.02</v>
       </c>
       <c r="F27" s="5" t="n">
-        <v>0.54</v>
+        <v>0.28</v>
       </c>
       <c r="G27" s="5" t="n">
-        <v>1.08</v>
+        <v>2.06</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>87.2</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="I27" s="7" t="n">
-        <v>4.147592651637327e-05</v>
+        <v>0.0200088938545985</v>
       </c>
       <c r="J27" s="8" t="n">
-        <v>639823</v>
+        <v>508427</v>
       </c>
       <c r="K27" s="8" t="n">
-        <v>40922</v>
+        <v>63225</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>betaine</t>
+          <t>mediterranean_diet</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="C28" s="5" t="n">
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>1.07</v>
+        <v>0.83</v>
       </c>
       <c r="F28" s="5" t="n">
-        <v>0.02</v>
+        <v>0.54</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>37.25</v>
+        <v>1.08</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>81.90000000000001</v>
+        <v>87.2</v>
       </c>
       <c r="I28" s="7" t="n">
-        <v>0.1779303397630421</v>
+        <v>4.147592651637327e-05</v>
       </c>
       <c r="J28" s="8" t="n">
-        <v>77198</v>
+        <v>639823</v>
       </c>
       <c r="K28" s="8" t="n">
-        <v>5297</v>
+        <v>40922</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>cod_liver_oil</t>
+          <t>betaine</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29" s="5" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>0.68</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
+        <v>1.07</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>37.25</v>
+      </c>
       <c r="H29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" s="7" t="n"/>
+        <v>81.90000000000001</v>
+      </c>
+      <c r="I29" s="7" t="n">
+        <v>0.1779303397630421</v>
+      </c>
       <c r="J29" s="8" t="n">
-        <v>4001</v>
+        <v>77198</v>
       </c>
       <c r="K29" s="8" t="n">
-        <v>1731</v>
+        <v>5297</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>iodine</t>
+          <t>cod_liver_oil</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>0.78</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>0.6</v>
+        <v>0.68</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.99</v>
+        <v>0.9</v>
       </c>
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="5" t="n"/>
@@ -1524,232 +1518,232 @@
       </c>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="8" t="n">
-        <v>2295</v>
+        <v>4001</v>
       </c>
       <c r="K30" s="8" t="n">
-        <v>1159</v>
+        <v>1731</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>folic_acid</t>
+          <t>iodine</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>37</v>
+        <v>1</v>
       </c>
       <c r="C31" s="5" t="n">
-        <v>0.8</v>
+        <v>0.78</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>0.73</v>
+        <v>0.6</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.89</v>
-      </c>
-      <c r="F31" s="5" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="G31" s="5" t="n">
-        <v>1.36</v>
-      </c>
+        <v>0.99</v>
+      </c>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
       <c r="H31" s="6" t="n">
-        <v>81.59999999999999</v>
-      </c>
-      <c r="I31" s="7" t="n">
-        <v>0.002768602416666183</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I31" s="7" t="n"/>
       <c r="J31" s="8" t="n">
-        <v>1078947</v>
+        <v>2295</v>
       </c>
       <c r="K31" s="8" t="n">
-        <v>52167</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>miso</t>
+          <t>folic_acid</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="C32" s="5" t="n">
         <v>0.8</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.73</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>1.13</v>
+        <v>0.89</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.02</v>
+        <v>0.47</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>33.61</v>
+        <v>1.36</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>57</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>0.5607534123225348</v>
+        <v>0.002768602416666183</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>87065</v>
+        <v>1078947</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>751</v>
+        <v>52167</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>vitamin_d</t>
+          <t>miso</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>75</v>
+        <v>3</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0.79</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>0.86</v>
+        <v>1.13</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.61</v>
+        <v>0.02</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>1.11</v>
+        <v>33.61</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>83.8</v>
+        <v>57</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>5.261486437358412e-08</v>
+        <v>0.5607534123225348</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>1315839</v>
+        <v>87065</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>99816</v>
+        <v>751</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>vitamin_e</t>
+          <t>fermented_foods</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>0.82</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>0.68</v>
+        <v>0.65</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>0.97</v>
+        <v>1.04</v>
       </c>
       <c r="F34" s="5" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="G34" s="5" t="n">
-        <v>1.77</v>
+        <v>1.91</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>84.5</v>
+        <v>90.8</v>
       </c>
       <c r="I34" s="7" t="n">
-        <v>0.094160471030461</v>
+        <v>0.5897124894853759</v>
       </c>
       <c r="J34" s="8" t="n">
-        <v>328582</v>
+        <v>190614</v>
       </c>
       <c r="K34" s="8" t="n">
-        <v>33305</v>
+        <v>42598</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>yogurt</t>
+          <t>vitamin_d</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
-        <v>5</v>
+        <v>75</v>
       </c>
       <c r="C35" s="5" t="n">
         <v>0.82</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>0.73</v>
+        <v>0.79</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.86</v>
       </c>
       <c r="F35" s="5" t="n">
-        <v>0.57</v>
+        <v>0.61</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>1.2</v>
+        <v>1.11</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>58.7</v>
+        <v>83.8</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>0.03213831121723015</v>
+        <v>5.261486437358412e-08</v>
       </c>
       <c r="J35" s="8" t="n">
-        <v>20962</v>
+        <v>1315839</v>
       </c>
       <c r="K35" s="8" t="n">
-        <v>40377</v>
+        <v>99816</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>flax</t>
+          <t>yogurt</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C36" s="5" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>0.72</v>
+        <v>0.73</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>1.2</v>
+      </c>
       <c r="H36" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="7" t="n"/>
+        <v>58.7</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>0.03213831121723015</v>
+      </c>
       <c r="J36" s="8" t="n">
-        <v>6369</v>
+        <v>20962</v>
       </c>
       <c r="K36" s="8" t="n">
-        <v>2999</v>
+        <v>40377</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>flaxseed</t>
+          <t>flax</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
@@ -1780,618 +1774,612 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>melatonin</t>
+          <t>flaxseed</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C38" s="5" t="n">
-        <v>0.85</v>
+        <v>0.84</v>
       </c>
       <c r="D38" s="5" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="5" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="G38" s="5" t="n">
-        <v>1.31</v>
-      </c>
+        <v>0.97</v>
+      </c>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
       <c r="H38" s="6" t="n">
-        <v>42.3</v>
-      </c>
-      <c r="I38" s="7" t="n">
-        <v>0.9864318175325136</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I38" s="7" t="n"/>
       <c r="J38" s="8" t="n">
-        <v>62422</v>
+        <v>6369</v>
       </c>
       <c r="K38" s="8" t="n">
-        <v>3175</v>
+        <v>2999</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>fermented_foods</t>
+          <t>manganese</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="C39" s="5" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="D39" s="5" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.73</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="F39" s="5" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G39" s="5" t="n">
-        <v>1.87</v>
-      </c>
+        <v>0.99</v>
+      </c>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
       <c r="H39" s="6" t="n">
-        <v>90.8</v>
-      </c>
-      <c r="I39" s="7" t="n">
-        <v>0.6093332948568936</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I39" s="7" t="n"/>
       <c r="J39" s="8" t="n">
-        <v>218102</v>
+        <v>2939</v>
       </c>
       <c r="K39" s="8" t="n">
-        <v>46171</v>
+        <v>382</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>green_tea</t>
+          <t>melatonin</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>0.89</v>
+        <v>0.85</v>
       </c>
       <c r="D40" s="5" t="n">
-        <v>0.77</v>
+        <v>0.73</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="F40" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>1.4</v>
+        <v>1.31</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>85.7</v>
+        <v>42.3</v>
       </c>
       <c r="I40" s="7" t="n">
-        <v>0.192122449317125</v>
+        <v>0.9864318175325136</v>
       </c>
       <c r="J40" s="8" t="n">
-        <v>274406</v>
+        <v>62422</v>
       </c>
       <c r="K40" s="8" t="n">
-        <v>18211</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>vitamin_a</t>
+          <t>vitamin_e</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C41" s="5" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="D41" s="5" t="n">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>1.09</v>
+        <v>1.01</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.43</v>
+        <v>0.42</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>1.88</v>
+        <v>1.69</v>
       </c>
       <c r="H41" s="6" t="n">
-        <v>87</v>
+        <v>81.8</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>0.5117296187637109</v>
+        <v>0.1288146566584174</v>
       </c>
       <c r="J41" s="8" t="n">
-        <v>322062</v>
+        <v>258436</v>
       </c>
       <c r="K41" s="8" t="n">
-        <v>20383</v>
+        <v>30662</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>calcium</t>
+          <t>green_tea</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C42" s="5" t="n">
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
       <c r="D42" s="5" t="n">
-        <v>0.86</v>
+        <v>0.77</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.96</v>
+        <v>1.02</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.76</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>1.08</v>
+        <v>1.4</v>
       </c>
       <c r="H42" s="6" t="n">
-        <v>81</v>
+        <v>85.7</v>
       </c>
       <c r="I42" s="7" t="n">
-        <v>0.02639264973927821</v>
+        <v>0.192122449317125</v>
       </c>
       <c r="J42" s="8" t="n">
-        <v>894018</v>
+        <v>274406</v>
       </c>
       <c r="K42" s="8" t="n">
-        <v>76477</v>
+        <v>18211</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>vitamin_c</t>
+          <t>vitamin_a</t>
         </is>
       </c>
       <c r="B43" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C43" s="5" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.9</v>
       </c>
       <c r="D43" s="5" t="n">
-        <v>0.82</v>
+        <v>0.74</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>1.06</v>
+        <v>1.09</v>
       </c>
       <c r="F43" s="5" t="n">
-        <v>0.59</v>
+        <v>0.43</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>1.48</v>
+        <v>1.88</v>
       </c>
       <c r="H43" s="6" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>0.5612991451474082</v>
+        <v>0.5117296187637109</v>
       </c>
       <c r="J43" s="8" t="n">
-        <v>512782</v>
+        <v>322062</v>
       </c>
       <c r="K43" s="8" t="n">
-        <v>35415</v>
+        <v>20383</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>selenium</t>
+          <t>calcium</t>
         </is>
       </c>
       <c r="B44" s="4" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C44" s="5" t="n">
-        <v>0.95</v>
+        <v>0.91</v>
       </c>
       <c r="D44" s="5" t="n">
-        <v>0.88</v>
+        <v>0.86</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>1.03</v>
+        <v>0.96</v>
       </c>
       <c r="F44" s="5" t="n">
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
       <c r="G44" s="5" t="n">
-        <v>1.22</v>
+        <v>1.08</v>
       </c>
       <c r="H44" s="6" t="n">
-        <v>58.4</v>
+        <v>81</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>0.8524602198215492</v>
+        <v>0.02639264973927821</v>
       </c>
       <c r="J44" s="8" t="n">
-        <v>346098</v>
+        <v>894018</v>
       </c>
       <c r="K44" s="8" t="n">
-        <v>21359</v>
+        <v>76477</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>caffeine</t>
+          <t>vitamin_c</t>
         </is>
       </c>
       <c r="B45" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C45" s="5" t="n">
-        <v>0.97</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="D45" s="5" t="n">
-        <v>0.92</v>
+        <v>0.82</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>1.01</v>
+        <v>1.06</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.85</v>
+        <v>0.59</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>1.1</v>
+        <v>1.48</v>
       </c>
       <c r="H45" s="6" t="n">
-        <v>45.9</v>
+        <v>83</v>
       </c>
       <c r="I45" s="7" t="n">
-        <v>0.4259906328747331</v>
+        <v>0.5612991451474082</v>
       </c>
       <c r="J45" s="8" t="n">
-        <v>872194</v>
+        <v>512782</v>
       </c>
       <c r="K45" s="8" t="n">
-        <v>38461</v>
+        <v>35415</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>dairy</t>
+          <t>selenium</t>
         </is>
       </c>
       <c r="B46" s="4" t="n">
-        <v>46</v>
+        <v>19</v>
       </c>
       <c r="C46" s="5" t="n">
-        <v>0.97</v>
+        <v>0.95</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>0.92</v>
+        <v>0.88</v>
       </c>
       <c r="E46" s="5" t="n">
         <v>1.03</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>1.27</v>
+        <v>1.22</v>
       </c>
       <c r="H46" s="6" t="n">
-        <v>84.3</v>
+        <v>58.4</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>0.240229660312519</v>
+        <v>0.8524602198215492</v>
       </c>
       <c r="J46" s="8" t="n">
-        <v>2055428</v>
+        <v>346098</v>
       </c>
       <c r="K46" s="8" t="n">
-        <v>92012</v>
+        <v>21359</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>bcaas</t>
+          <t>caffeine</t>
         </is>
       </c>
       <c r="B47" s="4" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="C47" s="5" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="D47" s="5" t="n">
-        <v>0.87</v>
+        <v>0.92</v>
       </c>
       <c r="E47" s="5" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F47" s="5" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G47" s="5" t="n">
         <v>1.1</v>
       </c>
-      <c r="F47" s="5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G47" s="5" t="n">
-        <v>3.8</v>
-      </c>
       <c r="H47" s="6" t="n">
-        <v>85.59999999999999</v>
+        <v>45.9</v>
       </c>
       <c r="I47" s="7" t="n">
-        <v>0.2941582730123437</v>
+        <v>0.4259906328747331</v>
       </c>
       <c r="J47" s="8" t="n">
-        <v>223922</v>
+        <v>872194</v>
       </c>
       <c r="K47" s="8" t="n">
-        <v>13868</v>
+        <v>38461</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>isoleucine</t>
+          <t>dairy</t>
         </is>
       </c>
       <c r="B48" s="4" t="n">
-        <v>4</v>
+        <v>46</v>
       </c>
       <c r="C48" s="5" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="D48" s="5" t="n">
-        <v>0.87</v>
+        <v>0.92</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>1.14</v>
+        <v>1.03</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>0.57</v>
+        <v>0.75</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>1.74</v>
+        <v>1.27</v>
       </c>
       <c r="H48" s="6" t="n">
-        <v>86.09999999999999</v>
+        <v>84.3</v>
       </c>
       <c r="I48" s="7" t="n">
-        <v>0.9376775415524352</v>
+        <v>0.240229660312519</v>
       </c>
       <c r="J48" s="8" t="n">
-        <v>227916</v>
+        <v>2055428</v>
       </c>
       <c r="K48" s="8" t="n">
-        <v>15865</v>
+        <v>92012</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>leucine</t>
+          <t>bcaas</t>
         </is>
       </c>
       <c r="B49" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C49" s="5" t="n">
-        <v>1.01</v>
+        <v>0.98</v>
       </c>
       <c r="D49" s="5" t="n">
-        <v>0.91</v>
+        <v>0.87</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>1.13</v>
+        <v>1.1</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>0.65</v>
+        <v>0.25</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>1.57</v>
+        <v>3.8</v>
       </c>
       <c r="H49" s="6" t="n">
-        <v>80.8</v>
+        <v>85.59999999999999</v>
       </c>
       <c r="I49" s="7" t="n">
-        <v>0.5613202208181812</v>
+        <v>0.2941582730123437</v>
       </c>
       <c r="J49" s="8" t="n">
-        <v>225687</v>
+        <v>223922</v>
       </c>
       <c r="K49" s="8" t="n">
-        <v>15633</v>
+        <v>13868</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>magnesium</t>
+          <t>isoleucine</t>
         </is>
       </c>
       <c r="B50" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C50" s="5" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="D50" s="5" t="n">
-        <v>0.8</v>
+        <v>0.87</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>1.29</v>
+        <v>1.14</v>
       </c>
       <c r="F50" s="5" t="n">
-        <v>0.06</v>
+        <v>0.57</v>
       </c>
       <c r="G50" s="5" t="n">
-        <v>15.95</v>
+        <v>1.74</v>
       </c>
       <c r="H50" s="6" t="n">
-        <v>79.8</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="I50" s="7" t="n">
-        <v>0.8073423351700231</v>
+        <v>0.9376775415524352</v>
       </c>
       <c r="J50" s="8" t="n">
-        <v>69780</v>
+        <v>227916</v>
       </c>
       <c r="K50" s="8" t="n">
-        <v>9994</v>
+        <v>15865</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>manganese</t>
+          <t>leucine</t>
         </is>
       </c>
       <c r="B51" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C51" s="5" t="n">
         <v>1.01</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>0.73</v>
+        <v>0.91</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F51" s="5" t="n"/>
-      <c r="G51" s="5" t="n"/>
+        <v>1.13</v>
+      </c>
+      <c r="F51" s="5" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G51" s="5" t="n">
+        <v>1.57</v>
+      </c>
       <c r="H51" s="6" t="n">
-        <v>94.40000000000001</v>
-      </c>
-      <c r="I51" s="7" t="n"/>
+        <v>80.8</v>
+      </c>
+      <c r="I51" s="7" t="n">
+        <v>0.5613202208181812</v>
+      </c>
       <c r="J51" s="8" t="n">
-        <v>225520</v>
+        <v>225687</v>
       </c>
       <c r="K51" s="8" t="n">
-        <v>29318</v>
+        <v>15633</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>tea</t>
+          <t>magnesium</t>
         </is>
       </c>
       <c r="B52" s="4" t="n">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="C52" s="5" t="n">
         <v>1.01</v>
       </c>
       <c r="D52" s="5" t="n">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>1.11</v>
+        <v>1.29</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0.66</v>
+        <v>0.06</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>1.53</v>
+        <v>15.95</v>
       </c>
       <c r="H52" s="6" t="n">
-        <v>91.09999999999999</v>
+        <v>79.8</v>
       </c>
       <c r="I52" s="7" t="n">
-        <v>0.894943683890389</v>
+        <v>0.8073423351700231</v>
       </c>
       <c r="J52" s="8" t="n">
-        <v>1206930</v>
+        <v>69780</v>
       </c>
       <c r="K52" s="8" t="n">
-        <v>65930</v>
+        <v>9994</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>vitamin_k</t>
+          <t>tea</t>
         </is>
       </c>
       <c r="B53" s="4" t="n">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="C53" s="5" t="n">
         <v>1.01</v>
       </c>
       <c r="D53" s="5" t="n">
-        <v>0.68</v>
+        <v>0.92</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F53" s="5" t="n"/>
-      <c r="G53" s="5" t="n"/>
+        <v>1.11</v>
+      </c>
+      <c r="F53" s="5" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G53" s="5" t="n">
+        <v>1.53</v>
+      </c>
       <c r="H53" s="6" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="I53" s="7" t="n"/>
+        <v>91.09999999999999</v>
+      </c>
+      <c r="I53" s="7" t="n">
+        <v>0.894943683890389</v>
+      </c>
       <c r="J53" s="8" t="n">
-        <v>5048</v>
+        <v>1206930</v>
       </c>
       <c r="K53" s="8" t="n">
-        <v>2592</v>
+        <v>65930</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>coenzyme_q10</t>
+          <t>vitamin_k</t>
         </is>
       </c>
       <c r="B54" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C54" s="5" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="D54" s="5" t="n">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>1.48</v>
-      </c>
-      <c r="F54" s="5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G54" s="5" t="n">
-        <v>5.18</v>
-      </c>
+        <v>1.5</v>
+      </c>
+      <c r="F54" s="5" t="n"/>
+      <c r="G54" s="5" t="n"/>
       <c r="H54" s="6" t="n">
-        <v>80.59999999999999</v>
-      </c>
-      <c r="I54" s="7" t="n">
-        <v>0.727583200950658</v>
-      </c>
+        <v>91.8</v>
+      </c>
+      <c r="I54" s="7" t="n"/>
       <c r="J54" s="8" t="n">
-        <v>581814</v>
+        <v>5048</v>
       </c>
       <c r="K54" s="8" t="n">
-        <v>75889</v>
+        <v>2592</v>
       </c>
     </row>
     <row r="55">
@@ -2533,495 +2521,489 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>grape</t>
+          <t>grapefruit</t>
         </is>
       </c>
       <c r="B59" s="4" t="n">
         <v>2</v>
       </c>
       <c r="C59" s="5" t="n">
-        <v>1.08</v>
+        <v>1.1</v>
       </c>
       <c r="D59" s="5" t="n">
-        <v>0.36</v>
+        <v>0.8</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>3.21</v>
+        <v>1.52</v>
       </c>
       <c r="F59" s="5" t="n"/>
       <c r="G59" s="5" t="n"/>
       <c r="H59" s="6" t="n">
-        <v>89.3</v>
+        <v>82.8</v>
       </c>
       <c r="I59" s="7" t="n"/>
       <c r="J59" s="8" t="n">
-        <v>1816</v>
+        <v>164504</v>
       </c>
       <c r="K59" s="8" t="n">
-        <v>609</v>
+        <v>5404</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>grapefruit</t>
+          <t>creatine</t>
         </is>
       </c>
       <c r="B60" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" s="5" t="n">
-        <v>1.1</v>
+        <v>1.11</v>
       </c>
       <c r="D60" s="5" t="n">
-        <v>0.8</v>
+        <v>1.01</v>
       </c>
       <c r="E60" s="5" t="n">
-        <v>1.52</v>
+        <v>1.19</v>
       </c>
       <c r="F60" s="5" t="n"/>
       <c r="G60" s="5" t="n"/>
       <c r="H60" s="6" t="n">
-        <v>82.8</v>
+        <v>0</v>
       </c>
       <c r="I60" s="7" t="n"/>
       <c r="J60" s="8" t="n">
-        <v>164504</v>
+        <v>207</v>
       </c>
       <c r="K60" s="8" t="n">
-        <v>5404</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>creatine</t>
+          <t>chromium</t>
         </is>
       </c>
       <c r="B61" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C61" s="5" t="n">
-        <v>1.11</v>
+        <v>1.13</v>
       </c>
       <c r="D61" s="5" t="n">
-        <v>1.01</v>
+        <v>1.06</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="F61" s="5" t="n"/>
-      <c r="G61" s="5" t="n"/>
+        <v>1.21</v>
+      </c>
+      <c r="F61" s="5" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G61" s="5" t="n">
+        <v>1.74</v>
+      </c>
       <c r="H61" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I61" s="7" t="n"/>
+      <c r="I61" s="7" t="n">
+        <v>0.9877864190999566</v>
+      </c>
       <c r="J61" s="8" t="n">
-        <v>207</v>
+        <v>66508</v>
       </c>
       <c r="K61" s="8" t="n">
-        <v>1057</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>chromium</t>
+          <t>glutamine</t>
         </is>
       </c>
       <c r="B62" s="4" t="n">
         <v>3</v>
       </c>
       <c r="C62" s="5" t="n">
-        <v>1.13</v>
+        <v>1.14</v>
       </c>
       <c r="D62" s="5" t="n">
-        <v>1.06</v>
+        <v>0.8</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>1.21</v>
+        <v>1.63</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>0.74</v>
+        <v>0.01</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>1.74</v>
+        <v>93.62</v>
       </c>
       <c r="H62" s="6" t="n">
-        <v>0</v>
+        <v>91.5</v>
       </c>
       <c r="I62" s="7" t="n">
-        <v>0.9877864190999566</v>
+        <v>0.214434325667662</v>
       </c>
       <c r="J62" s="8" t="n">
-        <v>66508</v>
+        <v>4702</v>
       </c>
       <c r="K62" s="8" t="n">
-        <v>1506</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>glutamine</t>
+          <t>zinc</t>
         </is>
       </c>
       <c r="B63" s="4" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="C63" s="5" t="n">
         <v>1.14</v>
       </c>
       <c r="D63" s="5" t="n">
-        <v>0.8</v>
+        <v>0.68</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>1.63</v>
+        <v>1.91</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>0.01</v>
+        <v>0.16</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>93.62</v>
+        <v>8.09</v>
       </c>
       <c r="H63" s="6" t="n">
-        <v>91.5</v>
+        <v>96</v>
       </c>
       <c r="I63" s="7" t="n">
-        <v>0.214434325667662</v>
+        <v>0.6073544042976849</v>
       </c>
       <c r="J63" s="8" t="n">
-        <v>4702</v>
+        <v>119440</v>
       </c>
       <c r="K63" s="8" t="n">
-        <v>2112</v>
+        <v>10103</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>zinc</t>
+          <t>iron</t>
         </is>
       </c>
       <c r="B64" s="4" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C64" s="5" t="n">
-        <v>1.14</v>
+        <v>1.15</v>
       </c>
       <c r="D64" s="5" t="n">
-        <v>0.68</v>
+        <v>1.05</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>1.91</v>
+        <v>1.25</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>0.16</v>
+        <v>0.83</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>8.09</v>
+        <v>1.6</v>
       </c>
       <c r="H64" s="6" t="n">
-        <v>96</v>
+        <v>81.2</v>
       </c>
       <c r="I64" s="7" t="n">
-        <v>0.6073544042976849</v>
+        <v>0.1931423553808725</v>
       </c>
       <c r="J64" s="8" t="n">
-        <v>119440</v>
+        <v>1147263</v>
       </c>
       <c r="K64" s="8" t="n">
-        <v>10103</v>
+        <v>98457</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>iron</t>
+          <t>eggs</t>
         </is>
       </c>
       <c r="B65" s="4" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C65" s="5" t="n">
-        <v>1.15</v>
+        <v>1.19</v>
       </c>
       <c r="D65" s="5" t="n">
-        <v>1.05</v>
+        <v>0.99</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>1.25</v>
+        <v>1.43</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>0.83</v>
+        <v>0.7</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>1.6</v>
+        <v>2.02</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>81.2</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>0.1931423553808725</v>
+        <v>0.9936223155021582</v>
       </c>
       <c r="J65" s="8" t="n">
-        <v>1147263</v>
+        <v>29311</v>
       </c>
       <c r="K65" s="8" t="n">
-        <v>98457</v>
+        <v>5421</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>eggs</t>
+          <t>alcohol</t>
         </is>
       </c>
       <c r="B66" s="4" t="n">
-        <v>8</v>
+        <v>203</v>
       </c>
       <c r="C66" s="5" t="n">
-        <v>1.19</v>
+        <v>1.27</v>
       </c>
       <c r="D66" s="5" t="n">
-        <v>0.99</v>
+        <v>1.24</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>1.43</v>
+        <v>1.29</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>0.7</v>
+        <v>1.05</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>2.02</v>
+        <v>1.53</v>
       </c>
       <c r="H66" s="6" t="n">
-        <v>86.90000000000001</v>
+        <v>90.2</v>
       </c>
       <c r="I66" s="7" t="n">
-        <v>0.9936223155021582</v>
+        <v>7.90723755922392e-33</v>
       </c>
       <c r="J66" s="8" t="n">
-        <v>29311</v>
+        <v>16471419</v>
       </c>
       <c r="K66" s="8" t="n">
-        <v>5421</v>
+        <v>1313337</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>alcohol</t>
+          <t>red_meat</t>
         </is>
       </c>
       <c r="B67" s="4" t="n">
-        <v>203</v>
+        <v>35</v>
       </c>
       <c r="C67" s="5" t="n">
         <v>1.27</v>
       </c>
       <c r="D67" s="5" t="n">
-        <v>1.24</v>
+        <v>1.2</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1.29</v>
+        <v>1.34</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>1.05</v>
+        <v>1</v>
       </c>
       <c r="G67" s="5" t="n">
-        <v>1.53</v>
+        <v>1.61</v>
       </c>
       <c r="H67" s="6" t="n">
-        <v>90.2</v>
+        <v>88.3</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>7.90723755922392e-33</v>
+        <v>1.319761565701576e-10</v>
       </c>
       <c r="J67" s="8" t="n">
-        <v>16471419</v>
+        <v>1260095</v>
       </c>
       <c r="K67" s="8" t="n">
-        <v>1313337</v>
+        <v>70729</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>red_meat</t>
+          <t>dehydroepiandrosterone</t>
         </is>
       </c>
       <c r="B68" s="4" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="C68" s="5" t="n">
-        <v>1.27</v>
+        <v>1.29</v>
       </c>
       <c r="D68" s="5" t="n">
-        <v>1.2</v>
+        <v>1.17</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>1.34</v>
+        <v>1.41</v>
       </c>
       <c r="F68" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>1.61</v>
+        <v>1.66</v>
       </c>
       <c r="H68" s="6" t="n">
-        <v>88.3</v>
+        <v>51.1</v>
       </c>
       <c r="I68" s="7" t="n">
-        <v>1.319761565701576e-10</v>
+        <v>0.0009428631078015041</v>
       </c>
       <c r="J68" s="8" t="n">
-        <v>1260095</v>
+        <v>20445</v>
       </c>
       <c r="K68" s="8" t="n">
-        <v>70729</v>
+        <v>4546</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>dehydroepiandrosterone</t>
+          <t>cannabidiol</t>
         </is>
       </c>
       <c r="B69" s="4" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C69" s="5" t="n">
-        <v>1.29</v>
+        <v>1.4</v>
       </c>
       <c r="D69" s="5" t="n">
-        <v>1.17</v>
+        <v>1.39</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="F69" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G69" s="5" t="n">
-        <v>1.66</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="F69" s="5" t="n"/>
+      <c r="G69" s="5" t="n"/>
       <c r="H69" s="6" t="n">
-        <v>51.1</v>
-      </c>
-      <c r="I69" s="7" t="n">
-        <v>0.0009428631078015041</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I69" s="7" t="n"/>
       <c r="J69" s="8" t="n">
-        <v>20445</v>
+        <v>124896418350</v>
       </c>
       <c r="K69" s="8" t="n">
-        <v>4546</v>
+        <v>51623922</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>cannabidiol</t>
+          <t>copper</t>
         </is>
       </c>
       <c r="B70" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C70" s="5" t="n">
-        <v>1.4</v>
+        <v>1.66</v>
       </c>
       <c r="D70" s="5" t="n">
-        <v>1.39</v>
+        <v>1.07</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F70" s="5" t="n"/>
-      <c r="G70" s="5" t="n"/>
+        <v>2.56</v>
+      </c>
+      <c r="F70" s="5" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="G70" s="5" t="n">
+        <v>7.5</v>
+      </c>
       <c r="H70" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I70" s="7" t="n"/>
+        <v>89</v>
+      </c>
+      <c r="I70" s="7" t="n">
+        <v>0.4612984675749361</v>
+      </c>
       <c r="J70" s="8" t="n">
-        <v>124896418350</v>
+        <v>65747</v>
       </c>
       <c r="K70" s="8" t="n">
-        <v>51623922</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>copper</t>
+          <t>omega-6_fatty_acids</t>
         </is>
       </c>
       <c r="B71" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C71" s="5" t="n">
-        <v>1.66</v>
+        <v>1.74</v>
       </c>
       <c r="D71" s="5" t="n">
-        <v>1.07</v>
+        <v>1.26</v>
       </c>
       <c r="E71" s="5" t="n">
-        <v>2.56</v>
-      </c>
-      <c r="F71" s="5" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="G71" s="5" t="n">
-        <v>7.5</v>
-      </c>
+        <v>2.42</v>
+      </c>
+      <c r="F71" s="5" t="n"/>
+      <c r="G71" s="5" t="n"/>
       <c r="H71" s="6" t="n">
-        <v>89</v>
-      </c>
-      <c r="I71" s="7" t="n">
-        <v>0.4612984675749361</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I71" s="7" t="n"/>
       <c r="J71" s="8" t="n">
-        <v>65747</v>
+        <v>2476</v>
       </c>
       <c r="K71" s="8" t="n">
-        <v>1930</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>omega-6_fatty_acids</t>
+          <t>coenzyme_q10</t>
         </is>
       </c>
       <c r="B72" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C72" s="5" t="n">
-        <v>1.88</v>
+        <v>1.94</v>
       </c>
       <c r="D72" s="5" t="n">
-        <v>1.41</v>
+        <v>1.19</v>
       </c>
       <c r="E72" s="5" t="n">
-        <v>2.51</v>
-      </c>
-      <c r="F72" s="5" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="G72" s="5" t="n">
-        <v>12.25</v>
-      </c>
+        <v>2.96</v>
+      </c>
+      <c r="F72" s="5" t="n"/>
+      <c r="G72" s="5" t="n"/>
       <c r="H72" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="I72" s="7" t="n">
-        <v>0.3558547673635933</v>
-      </c>
+      <c r="I72" s="7" t="n"/>
       <c r="J72" s="8" t="n">
-        <v>3160</v>
+        <v>449</v>
       </c>
       <c r="K72" s="8" t="n">
-        <v>1518</v>
+        <v>160</v>
       </c>
     </row>
     <row r="73">

</xml_diff>

<commit_message>
Refresh localized folic acid figures
</commit_message>
<xml_diff>
--- a/Plot/exposures_meta_analysis_breast_combined.xlsx
+++ b/Plot/exposures_meta_analysis_breast_combined.xlsx
@@ -1558,75 +1558,75 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>folic_acid</t>
+          <t>miso</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="C32" s="5" t="n">
         <v>0.8</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>0.73</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.89</v>
+        <v>1.13</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.47</v>
+        <v>0.02</v>
       </c>
       <c r="G32" s="5" t="n">
-        <v>1.36</v>
+        <v>33.61</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>81.59999999999999</v>
+        <v>57</v>
       </c>
       <c r="I32" s="7" t="n">
-        <v>0.002768602416666183</v>
+        <v>0.5607534123225348</v>
       </c>
       <c r="J32" s="8" t="n">
-        <v>1078947</v>
+        <v>87065</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>52167</v>
+        <v>751</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>miso</t>
+          <t>folic_acid</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="C33" s="5" t="n">
-        <v>0.8</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.73</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>1.13</v>
+        <v>0.9</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.02</v>
+        <v>0.48</v>
       </c>
       <c r="G33" s="5" t="n">
-        <v>33.61</v>
+        <v>1.37</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>57</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="I33" s="7" t="n">
-        <v>0.5607534123225348</v>
+        <v>0.004484947230008314</v>
       </c>
       <c r="J33" s="8" t="n">
-        <v>87065</v>
+        <v>1076873</v>
       </c>
       <c r="K33" s="8" t="n">
-        <v>751</v>
+        <v>51167</v>
       </c>
     </row>
     <row r="34">

</xml_diff>